<commit_message>
Update BOM images and PCB page image review, and Index links
</commit_message>
<xml_diff>
--- a/docs/04-BOM/DirksBOM.xlsx
+++ b/docs/04-BOM/DirksBOM.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Precision\Desktop\J2DIndivGithub\Classwork\JacobDirksEGR314.github.io\docs\04-BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DD1A294F-4811-41D4-AF53-2EA6A489890B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{808078F8-CBCF-4D93-8AB6-9F921C4C75DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12165" yWindow="0" windowWidth="16635" windowHeight="15600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14400" yWindow="0" windowWidth="14400" windowHeight="15600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -897,7 +897,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -912,6 +912,9 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1254,13 +1257,13 @@
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="21.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="20.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.42578125" customWidth="1"/>
+    <col min="3" max="3" width="9.5703125" customWidth="1"/>
+    <col min="4" max="4" width="9.85546875" customWidth="1"/>
+    <col min="5" max="5" width="11.140625" customWidth="1"/>
+    <col min="6" max="6" width="11.85546875" customWidth="1"/>
     <col min="7" max="7" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="19.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.7109375" customWidth="1"/>
     <col min="9" max="10" width="16.140625" customWidth="1"/>
     <col min="11" max="11" width="9.28515625" customWidth="1"/>
     <col min="12" max="12" width="12.42578125" customWidth="1"/>
@@ -1292,56 +1295,56 @@
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
     </row>
-    <row r="2" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:17" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="G2" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="H2" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="I2" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="J2" s="3" t="s">
+      <c r="J2" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="K2" s="3" t="s">
+      <c r="K2" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="L2" s="3" t="s">
+      <c r="L2" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="M2" s="3" t="s">
+      <c r="M2" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="N2" s="3" t="s">
+      <c r="N2" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="O2" s="3" t="s">
+      <c r="O2" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="P2" s="3" t="s">
+      <c r="P2" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="Q2" s="3" t="s">
+      <c r="Q2" s="12" t="s">
         <v>16</v>
       </c>
     </row>
@@ -3383,5 +3386,6 @@
     <hyperlink ref="J34" r:id="rId76" xr:uid="{B73BC35A-3897-4F61-B017-5964ACFB946C}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="landscape" r:id="rId77"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update PCB information after building and add images
</commit_message>
<xml_diff>
--- a/docs/04-BOM/DirksBOM.xlsx
+++ b/docs/04-BOM/DirksBOM.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Precision\Desktop\J2DIndivGithub\Classwork\JacobDirksEGR314.github.io\docs\04-BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{808078F8-CBCF-4D93-8AB6-9F921C4C75DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F8DE1B05-88A8-46B0-A537-42ABD2638B66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14400" yWindow="0" windowWidth="14400" windowHeight="15600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="14400" windowHeight="15600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="262">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="335" uniqueCount="273">
   <si>
     <t>Part Name/Description</t>
   </si>
@@ -458,15 +458,6 @@
     <t>FIXED IND 4.7UH 2.5A 147.2 MOHM</t>
   </si>
   <si>
-    <t>TDK</t>
-  </si>
-  <si>
-    <t>SPM4020T-4R7M-LR</t>
-  </si>
-  <si>
-    <t>445-174477-1-ND</t>
-  </si>
-  <si>
     <t>FIXED IND 33UH 2.5A 93.6 MOHM</t>
   </si>
   <si>
@@ -650,9 +641,6 @@
     <t xml:space="preserve">https://www.digikey.com/en/products/detail/schurter-inc/0034-3123/639683 </t>
   </si>
   <si>
-    <t xml:space="preserve">https://www.digikey.com/en/products/detail/tdk-corporation/SPM4020T-4R7M-LR/5962341 </t>
-  </si>
-  <si>
     <t xml:space="preserve">https://www.digikey.com/en/products/detail/murata-electronics/1274AS-H-330M-P3/5271492 </t>
   </si>
   <si>
@@ -743,9 +731,6 @@
     <t xml:space="preserve">https://www.schurter.com/en/datasheet/typ_FST_5x20.pdf </t>
   </si>
   <si>
-    <t xml:space="preserve">https://product.tdk.com/en/system/files?file=dam/doc/product/inductor/inductor/smd/catalog/inductor_commercial_power_spm4020-lr_en.pdf </t>
-  </si>
-  <si>
     <t xml:space="preserve">https://search.murata.co.jp/Ceramy/image/img/P02/J(E)TE243B-0058_DEM10050C_reference.pdf </t>
   </si>
   <si>
@@ -819,6 +804,54 @@
   </si>
   <si>
     <t>2223-TS02-66-55-BK-100-LCR-D-ND</t>
+  </si>
+  <si>
+    <t>RES SMD 196K OHM 1% 1/4W 0805</t>
+  </si>
+  <si>
+    <t>Vishay Dale</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/vishay-dale/CRCW0805196KFKEA/1175896</t>
+  </si>
+  <si>
+    <t>https://www.vishay.com/docs/20035/dcrcwe3.pdf</t>
+  </si>
+  <si>
+    <t>541-196KCCT-ND</t>
+  </si>
+  <si>
+    <t>R12</t>
+  </si>
+  <si>
+    <t>R8</t>
+  </si>
+  <si>
+    <t>RES 62K OHM 5% 1/8W 0805</t>
+  </si>
+  <si>
+    <t>RC0805JR-0762KL</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/yageo/RC0805JR-0762KL/728360</t>
+  </si>
+  <si>
+    <t>311-62KARDKR-ND</t>
+  </si>
+  <si>
+    <t>https://yageogroup.com/content/datasheet/asset/file/PYU-RC_GROUP_51_ROHS_L</t>
+  </si>
+  <si>
+    <t>NRS4018T6R8MDGJ</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/taiyo-yuden/NRS4018T6R8MDGJ/2648972</t>
+  </si>
+  <si>
+    <t>https://mm.digikey.com/Volume0/opasdata/d220001/medias/docus/7087/NR-H-S-V%20Datasheet.pdf</t>
+  </si>
+  <si>
+    <t>587-2894-6-ND</t>
   </si>
 </sst>
 </file>
@@ -869,7 +902,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -892,16 +925,23 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -915,6 +955,12 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1253,7 +1299,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:Q41"/>
+  <dimension ref="A1:Q43"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="21.7109375" bestFit="1" customWidth="1"/>
@@ -1262,7 +1308,7 @@
     <col min="4" max="4" width="9.85546875" customWidth="1"/>
     <col min="5" max="5" width="11.140625" customWidth="1"/>
     <col min="6" max="6" width="11.85546875" customWidth="1"/>
-    <col min="7" max="7" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.140625" customWidth="1"/>
     <col min="8" max="8" width="19.7109375" customWidth="1"/>
     <col min="9" max="10" width="16.140625" customWidth="1"/>
     <col min="11" max="11" width="9.28515625" customWidth="1"/>
@@ -1275,2032 +1321,2439 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="1" t="s">
-        <v>248</v>
-      </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
-      <c r="I1" s="2"/>
-      <c r="J1" s="2"/>
-      <c r="K1" s="2"/>
-      <c r="L1" s="2"/>
-      <c r="M1" s="2"/>
-      <c r="N1" s="2"/>
-      <c r="O1" s="2"/>
-      <c r="P1" s="2"/>
-      <c r="Q1" s="2"/>
+      <c r="A1" s="11" t="s">
+        <v>243</v>
+      </c>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="12"/>
+      <c r="H1" s="12"/>
+      <c r="I1" s="12"/>
+      <c r="J1" s="12"/>
+      <c r="K1" s="12"/>
+      <c r="L1" s="12"/>
+      <c r="M1" s="12"/>
+      <c r="N1" s="12"/>
+      <c r="O1" s="12"/>
+      <c r="P1" s="12"/>
+      <c r="Q1" s="12"/>
     </row>
     <row r="2" spans="1:17" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A2" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="12" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" s="12" t="s">
+      <c r="A2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="12" t="s">
+      <c r="D2" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="12" t="s">
+      <c r="E2" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="12" t="s">
+      <c r="F2" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G2" s="12" t="s">
+      <c r="G2" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="H2" s="12" t="s">
+      <c r="H2" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="I2" s="12" t="s">
+      <c r="I2" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="J2" s="12" t="s">
+      <c r="J2" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="K2" s="12" t="s">
+      <c r="K2" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="L2" s="12" t="s">
+      <c r="L2" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="M2" s="12" t="s">
+      <c r="M2" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="N2" s="12" t="s">
+      <c r="N2" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="O2" s="12" t="s">
+      <c r="O2" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="P2" s="12" t="s">
+      <c r="P2" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="Q2" s="12" t="s">
+      <c r="Q2" s="10" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="3" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B3" s="5">
-        <v>1</v>
-      </c>
-      <c r="C3" s="6">
+      <c r="B3" s="3">
+        <v>1</v>
+      </c>
+      <c r="C3" s="4">
         <v>5.49</v>
       </c>
-      <c r="D3" s="6">
-        <f t="shared" ref="D3:D38" si="0">B3*C3</f>
+      <c r="D3" s="4">
+        <f t="shared" ref="D3:D40" si="0">B3*C3</f>
         <v>5.49</v>
       </c>
-      <c r="E3" s="6">
+      <c r="E3" s="4">
         <f>C3</f>
         <v>5.49</v>
       </c>
-      <c r="F3" s="6">
-        <f t="shared" ref="F3:F38" si="1">B3*E3</f>
+      <c r="F3" s="4">
+        <f t="shared" ref="F3:F40" si="1">B3*E3</f>
         <v>5.49</v>
       </c>
-      <c r="G3" s="4" t="s">
+      <c r="G3" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="H3" s="4" t="s">
+      <c r="H3" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="I3" s="10" t="s">
-        <v>182</v>
-      </c>
-      <c r="J3" s="10" t="s">
-        <v>217</v>
-      </c>
-      <c r="K3" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="L3" s="4" t="s">
+      <c r="I3" s="8" t="s">
+        <v>179</v>
+      </c>
+      <c r="J3" s="8" t="s">
+        <v>213</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="L3" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="M3" s="4"/>
-      <c r="N3" s="7"/>
-      <c r="O3" s="4"/>
-      <c r="P3" s="5">
-        <f t="shared" ref="P3:P40" si="2">O3-B3</f>
-        <v>-1</v>
-      </c>
-      <c r="Q3" s="4" t="s">
+      <c r="M3" s="3">
+        <v>3</v>
+      </c>
+      <c r="N3" s="5">
+        <v>46093</v>
+      </c>
+      <c r="O3" s="3">
+        <f>M3</f>
+        <v>3</v>
+      </c>
+      <c r="P3" s="3">
+        <f t="shared" ref="P3:P42" si="2">O3-B3</f>
+        <v>2</v>
+      </c>
+      <c r="Q3" s="2" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="4" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="B4" s="8">
+      <c r="B4" s="6">
         <v>2</v>
       </c>
-      <c r="C4" s="6">
+      <c r="C4" s="4">
         <v>0.1</v>
       </c>
-      <c r="D4" s="6">
+      <c r="D4" s="4">
         <f t="shared" si="0"/>
         <v>0.2</v>
       </c>
-      <c r="E4" s="6">
-        <f t="shared" ref="E4:E38" si="3">C4</f>
+      <c r="E4" s="4">
+        <f t="shared" ref="E4:E40" si="3">C4</f>
         <v>0.1</v>
       </c>
-      <c r="F4" s="6">
+      <c r="F4" s="4">
         <f t="shared" si="1"/>
         <v>0.2</v>
       </c>
-      <c r="G4" s="4" t="s">
+      <c r="G4" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="H4" s="4" t="s">
+      <c r="H4" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="I4" s="10" t="s">
-        <v>183</v>
-      </c>
-      <c r="J4" s="10" t="s">
-        <v>218</v>
-      </c>
-      <c r="K4" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="L4" s="4" t="s">
+      <c r="I4" s="8" t="s">
+        <v>180</v>
+      </c>
+      <c r="J4" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="K4" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="L4" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="M4" s="4"/>
-      <c r="N4" s="7"/>
-      <c r="O4" s="4"/>
-      <c r="P4" s="5">
+      <c r="M4" s="2">
+        <v>2</v>
+      </c>
+      <c r="N4" s="5">
+        <f>N3</f>
+        <v>46093</v>
+      </c>
+      <c r="O4" s="3">
+        <f t="shared" ref="O4:O42" si="4">M4</f>
+        <v>2</v>
+      </c>
+      <c r="P4" s="3">
         <f>O4-B10</f>
-        <v>-2</v>
-      </c>
-      <c r="Q4" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="Q4" s="6" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="5" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="B5" s="5">
+      <c r="B5" s="3">
         <v>2</v>
       </c>
-      <c r="C5" s="6">
+      <c r="C5" s="4">
         <v>0.08</v>
       </c>
-      <c r="D5" s="6">
+      <c r="D5" s="4">
         <f t="shared" si="0"/>
         <v>0.16</v>
       </c>
-      <c r="E5" s="6">
+      <c r="E5" s="4">
         <f t="shared" si="3"/>
         <v>0.08</v>
       </c>
-      <c r="F5" s="6">
+      <c r="F5" s="4">
         <f t="shared" si="1"/>
         <v>0.16</v>
       </c>
-      <c r="G5" s="4" t="s">
+      <c r="G5" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="H5" s="4" t="s">
+      <c r="H5" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="I5" s="10" t="s">
-        <v>184</v>
-      </c>
-      <c r="J5" s="10" t="s">
-        <v>219</v>
-      </c>
-      <c r="K5" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="L5" s="4" t="s">
+      <c r="I5" s="8" t="s">
+        <v>181</v>
+      </c>
+      <c r="J5" s="8" t="s">
+        <v>215</v>
+      </c>
+      <c r="K5" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="L5" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="M5" s="4"/>
-      <c r="N5" s="7"/>
-      <c r="O5" s="4"/>
-      <c r="P5" s="5">
+      <c r="M5" s="2">
+        <v>1</v>
+      </c>
+      <c r="N5" s="5">
+        <f t="shared" ref="N5:N42" si="5">N4</f>
+        <v>46093</v>
+      </c>
+      <c r="O5" s="3">
+        <v>2</v>
+      </c>
+      <c r="P5" s="3">
         <f t="shared" si="2"/>
-        <v>-2</v>
-      </c>
-      <c r="Q5" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="Q5" s="6" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="6" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="B6" s="5">
-        <v>1</v>
-      </c>
-      <c r="C6" s="6">
+      <c r="B6" s="3">
+        <v>1</v>
+      </c>
+      <c r="C6" s="4">
         <v>0.1</v>
       </c>
-      <c r="D6" s="6">
+      <c r="D6" s="4">
         <f t="shared" si="0"/>
         <v>0.1</v>
       </c>
-      <c r="E6" s="6">
+      <c r="E6" s="4">
         <f t="shared" si="3"/>
         <v>0.1</v>
       </c>
-      <c r="F6" s="6">
+      <c r="F6" s="4">
         <f t="shared" si="1"/>
         <v>0.1</v>
       </c>
-      <c r="G6" s="4" t="s">
+      <c r="G6" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="H6" s="4" t="s">
+      <c r="H6" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="I6" s="10" t="s">
-        <v>185</v>
-      </c>
-      <c r="J6" s="10" t="s">
-        <v>220</v>
-      </c>
-      <c r="K6" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="L6" s="4" t="s">
+      <c r="I6" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="J6" s="8" t="s">
+        <v>216</v>
+      </c>
+      <c r="K6" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="L6" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="M6" s="4"/>
-      <c r="N6" s="7"/>
-      <c r="O6" s="8"/>
-      <c r="P6" s="5">
+      <c r="M6" s="2">
+        <v>1</v>
+      </c>
+      <c r="N6" s="5">
+        <f t="shared" si="5"/>
+        <v>46093</v>
+      </c>
+      <c r="O6" s="3">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="P6" s="3">
         <f t="shared" si="2"/>
-        <v>-1</v>
-      </c>
-      <c r="Q6" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="Q6" s="2" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="7" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="B7" s="5">
+      <c r="B7" s="3">
         <v>6</v>
       </c>
-      <c r="C7" s="6">
+      <c r="C7" s="4">
         <v>0.18</v>
       </c>
-      <c r="D7" s="6">
+      <c r="D7" s="4">
         <f t="shared" si="0"/>
         <v>1.08</v>
       </c>
-      <c r="E7" s="6">
+      <c r="E7" s="4">
         <f t="shared" si="3"/>
         <v>0.18</v>
       </c>
-      <c r="F7" s="6">
+      <c r="F7" s="4">
         <f t="shared" si="1"/>
         <v>1.08</v>
       </c>
-      <c r="G7" s="4" t="s">
+      <c r="G7" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="H7" s="4" t="s">
+      <c r="H7" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="I7" s="10" t="s">
-        <v>186</v>
-      </c>
-      <c r="J7" s="10" t="s">
-        <v>221</v>
-      </c>
-      <c r="K7" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="L7" s="4" t="s">
+      <c r="I7" s="8" t="s">
+        <v>183</v>
+      </c>
+      <c r="J7" s="8" t="s">
+        <v>217</v>
+      </c>
+      <c r="K7" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="L7" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="M7" s="4"/>
-      <c r="N7" s="7"/>
-      <c r="O7" s="8"/>
-      <c r="P7" s="5">
+      <c r="M7" s="2">
+        <v>1</v>
+      </c>
+      <c r="N7" s="5">
+        <f t="shared" si="5"/>
+        <v>46093</v>
+      </c>
+      <c r="O7" s="3">
+        <v>6</v>
+      </c>
+      <c r="P7" s="3">
         <f t="shared" si="2"/>
-        <v>-6</v>
-      </c>
-      <c r="Q7" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="Q7" s="6" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="8" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A8" s="4" t="s">
+      <c r="A8" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="B8" s="5">
+      <c r="B8" s="3">
         <v>7</v>
       </c>
-      <c r="C8" s="6">
+      <c r="C8" s="4">
         <v>0.08</v>
       </c>
-      <c r="D8" s="6">
+      <c r="D8" s="4">
         <f t="shared" si="0"/>
         <v>0.56000000000000005</v>
       </c>
-      <c r="E8" s="6">
+      <c r="E8" s="4">
         <f t="shared" si="3"/>
         <v>0.08</v>
       </c>
-      <c r="F8" s="6">
+      <c r="F8" s="4">
         <f t="shared" si="1"/>
         <v>0.56000000000000005</v>
       </c>
-      <c r="G8" s="4" t="s">
+      <c r="G8" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="H8" s="4" t="s">
+      <c r="H8" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="I8" s="10" t="s">
-        <v>187</v>
-      </c>
-      <c r="J8" s="10" t="s">
-        <v>222</v>
-      </c>
-      <c r="K8" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="L8" s="4" t="s">
+      <c r="I8" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="J8" s="8" t="s">
+        <v>218</v>
+      </c>
+      <c r="K8" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="L8" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="M8" s="4"/>
-      <c r="N8" s="7"/>
-      <c r="O8" s="4"/>
-      <c r="P8" s="5">
+      <c r="M8" s="2">
+        <v>10</v>
+      </c>
+      <c r="N8" s="5">
+        <f t="shared" si="5"/>
+        <v>46093</v>
+      </c>
+      <c r="O8" s="3">
+        <f t="shared" si="4"/>
+        <v>10</v>
+      </c>
+      <c r="P8" s="3">
         <f t="shared" si="2"/>
-        <v>-7</v>
-      </c>
-      <c r="Q8" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="Q8" s="6" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="9" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A9" s="4" t="s">
+      <c r="A9" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="B9" s="5">
-        <v>1</v>
-      </c>
-      <c r="C9" s="6">
+      <c r="B9" s="3">
+        <v>1</v>
+      </c>
+      <c r="C9" s="4">
         <v>0.08</v>
       </c>
-      <c r="D9" s="6">
+      <c r="D9" s="4">
         <f t="shared" si="0"/>
         <v>0.08</v>
       </c>
-      <c r="E9" s="6">
+      <c r="E9" s="4">
         <f t="shared" si="3"/>
         <v>0.08</v>
       </c>
-      <c r="F9" s="6">
+      <c r="F9" s="4">
         <f t="shared" si="1"/>
         <v>0.08</v>
       </c>
-      <c r="G9" s="4" t="s">
+      <c r="G9" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="H9" s="4" t="s">
+      <c r="H9" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="I9" s="10" t="s">
-        <v>188</v>
-      </c>
-      <c r="J9" s="10" t="s">
-        <v>223</v>
-      </c>
-      <c r="K9" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="L9" s="4" t="s">
+      <c r="I9" s="8" t="s">
+        <v>185</v>
+      </c>
+      <c r="J9" s="8" t="s">
+        <v>219</v>
+      </c>
+      <c r="K9" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="L9" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="M9" s="4"/>
-      <c r="N9" s="7"/>
-      <c r="O9" s="4"/>
-      <c r="P9" s="5">
+      <c r="M9" s="2">
+        <v>1</v>
+      </c>
+      <c r="N9" s="5">
+        <f t="shared" si="5"/>
+        <v>46093</v>
+      </c>
+      <c r="O9" s="3">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="P9" s="3">
         <f t="shared" si="2"/>
-        <v>-1</v>
-      </c>
-      <c r="Q9" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="Q9" s="6" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="10" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A10" s="4" t="s">
+      <c r="A10" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="B10" s="5">
+      <c r="B10" s="3">
         <v>2</v>
       </c>
-      <c r="C10" s="6">
+      <c r="C10" s="4">
         <v>0.1</v>
       </c>
-      <c r="D10" s="6">
+      <c r="D10" s="4">
         <f t="shared" si="0"/>
         <v>0.2</v>
       </c>
-      <c r="E10" s="6">
+      <c r="E10" s="4">
         <f t="shared" si="3"/>
         <v>0.1</v>
       </c>
-      <c r="F10" s="6">
+      <c r="F10" s="4">
         <f t="shared" si="1"/>
         <v>0.2</v>
       </c>
-      <c r="G10" s="4" t="s">
+      <c r="G10" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="H10" s="8" t="s">
+      <c r="H10" s="6" t="s">
         <v>121</v>
       </c>
-      <c r="I10" s="10" t="s">
-        <v>189</v>
-      </c>
-      <c r="J10" s="10" t="s">
-        <v>224</v>
-      </c>
-      <c r="K10" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="L10" s="8" t="s">
+      <c r="I10" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="J10" s="8" t="s">
+        <v>220</v>
+      </c>
+      <c r="K10" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="L10" s="6" t="s">
         <v>122</v>
       </c>
-      <c r="M10" s="8"/>
-      <c r="N10" s="7"/>
-      <c r="O10" s="8"/>
-      <c r="P10" s="5">
+      <c r="M10" s="6">
+        <v>3</v>
+      </c>
+      <c r="N10" s="5">
+        <f t="shared" si="5"/>
+        <v>46093</v>
+      </c>
+      <c r="O10" s="3">
+        <f t="shared" si="4"/>
+        <v>3</v>
+      </c>
+      <c r="P10" s="3">
         <f t="shared" si="2"/>
-        <v>-2</v>
-      </c>
-      <c r="Q10" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="Q10" s="6" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="11" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="B11" s="5">
-        <v>1</v>
-      </c>
-      <c r="C11" s="6">
+      <c r="B11" s="3">
+        <v>1</v>
+      </c>
+      <c r="C11" s="4">
         <v>0.08</v>
       </c>
-      <c r="D11" s="6">
+      <c r="D11" s="4">
         <f t="shared" si="0"/>
         <v>0.08</v>
       </c>
-      <c r="E11" s="6">
+      <c r="E11" s="4">
         <f t="shared" si="3"/>
         <v>0.08</v>
       </c>
-      <c r="F11" s="6">
+      <c r="F11" s="4">
         <f t="shared" si="1"/>
         <v>0.08</v>
       </c>
-      <c r="G11" s="4" t="s">
+      <c r="G11" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="H11" s="8" t="s">
+      <c r="H11" s="6" t="s">
         <v>112</v>
       </c>
-      <c r="I11" s="11" t="s">
-        <v>190</v>
-      </c>
-      <c r="J11" s="10" t="s">
-        <v>225</v>
-      </c>
-      <c r="K11" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="L11" s="8" t="s">
+      <c r="I11" s="9" t="s">
+        <v>187</v>
+      </c>
+      <c r="J11" s="8" t="s">
+        <v>221</v>
+      </c>
+      <c r="K11" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="L11" s="6" t="s">
         <v>113</v>
       </c>
-      <c r="M11" s="8"/>
-      <c r="N11" s="7"/>
-      <c r="O11" s="8"/>
-      <c r="P11" s="5">
+      <c r="M11" s="6">
+        <v>1</v>
+      </c>
+      <c r="N11" s="5">
+        <f t="shared" si="5"/>
+        <v>46093</v>
+      </c>
+      <c r="O11" s="3">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="P11" s="3">
         <f t="shared" si="2"/>
-        <v>-1</v>
-      </c>
-      <c r="Q11" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="Q11" s="6" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="12" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A12" s="4" t="s">
+      <c r="A12" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="B12" s="5">
+      <c r="B12" s="3">
         <v>4</v>
       </c>
-      <c r="C12" s="6">
+      <c r="C12" s="4">
         <v>0.28000000000000003</v>
       </c>
-      <c r="D12" s="6">
+      <c r="D12" s="4">
         <f t="shared" si="0"/>
         <v>1.1200000000000001</v>
       </c>
-      <c r="E12" s="6">
+      <c r="E12" s="4">
         <f t="shared" si="3"/>
         <v>0.28000000000000003</v>
       </c>
-      <c r="F12" s="6">
+      <c r="F12" s="4">
         <f t="shared" si="1"/>
         <v>1.1200000000000001</v>
       </c>
-      <c r="G12" s="8" t="s">
+      <c r="G12" s="6" t="s">
         <v>101</v>
       </c>
-      <c r="H12" s="8" t="s">
+      <c r="H12" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="I12" s="10" t="s">
-        <v>191</v>
-      </c>
-      <c r="J12" s="10" t="s">
-        <v>226</v>
-      </c>
-      <c r="K12" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="L12" s="8" t="s">
+      <c r="I12" s="8" t="s">
+        <v>188</v>
+      </c>
+      <c r="J12" s="8" t="s">
+        <v>222</v>
+      </c>
+      <c r="K12" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="L12" s="6" t="s">
         <v>106</v>
       </c>
-      <c r="M12" s="8"/>
-      <c r="N12" s="7"/>
-      <c r="O12" s="8"/>
-      <c r="P12" s="5">
+      <c r="M12" s="6">
+        <v>6</v>
+      </c>
+      <c r="N12" s="5">
+        <f t="shared" si="5"/>
+        <v>46093</v>
+      </c>
+      <c r="O12" s="3">
+        <f t="shared" si="4"/>
+        <v>6</v>
+      </c>
+      <c r="P12" s="3">
         <f t="shared" si="2"/>
-        <v>-4</v>
-      </c>
-      <c r="Q12" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="Q12" s="6" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="13" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A13" s="4" t="s">
+      <c r="A13" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="B13" s="5">
+      <c r="B13" s="3">
         <v>5</v>
       </c>
-      <c r="C13" s="6">
+      <c r="C13" s="4">
         <v>1.74</v>
       </c>
-      <c r="D13" s="6">
+      <c r="D13" s="4">
         <f t="shared" si="0"/>
         <v>8.6999999999999993</v>
       </c>
-      <c r="E13" s="6">
+      <c r="E13" s="4">
         <f t="shared" si="3"/>
         <v>1.74</v>
       </c>
-      <c r="F13" s="6">
+      <c r="F13" s="4">
         <f t="shared" si="1"/>
         <v>8.6999999999999993</v>
       </c>
-      <c r="G13" s="4" t="s">
+      <c r="G13" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="H13" s="8" t="s">
+      <c r="H13" s="6" t="s">
         <v>138</v>
       </c>
-      <c r="I13" s="10" t="s">
-        <v>192</v>
-      </c>
-      <c r="J13" s="10" t="s">
-        <v>225</v>
-      </c>
-      <c r="K13" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="L13" s="8" t="s">
+      <c r="I13" s="8" t="s">
+        <v>189</v>
+      </c>
+      <c r="J13" s="8" t="s">
+        <v>221</v>
+      </c>
+      <c r="K13" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="L13" s="6" t="s">
         <v>139</v>
       </c>
-      <c r="M13" s="8"/>
-      <c r="N13" s="7"/>
-      <c r="O13" s="8"/>
-      <c r="P13" s="5">
+      <c r="M13" s="6">
+        <v>7</v>
+      </c>
+      <c r="N13" s="5">
+        <f t="shared" si="5"/>
+        <v>46093</v>
+      </c>
+      <c r="O13" s="3">
+        <f t="shared" si="4"/>
+        <v>7</v>
+      </c>
+      <c r="P13" s="3">
         <f t="shared" si="2"/>
-        <v>-5</v>
-      </c>
-      <c r="Q13" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="Q13" s="6" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="14" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A14" s="4" t="s">
+      <c r="A14" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="B14" s="5">
-        <v>1</v>
-      </c>
-      <c r="C14" s="6">
+      <c r="B14" s="3">
+        <v>1</v>
+      </c>
+      <c r="C14" s="4">
         <v>1.31</v>
       </c>
-      <c r="D14" s="6">
+      <c r="D14" s="4">
         <f t="shared" si="0"/>
         <v>1.31</v>
       </c>
-      <c r="E14" s="6">
+      <c r="E14" s="4">
         <f t="shared" si="3"/>
         <v>1.31</v>
       </c>
-      <c r="F14" s="6">
+      <c r="F14" s="4">
         <f t="shared" si="1"/>
         <v>1.31</v>
       </c>
-      <c r="G14" s="8" t="s">
+      <c r="G14" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="H14" s="8" t="s">
+      <c r="H14" s="6" t="s">
         <v>98</v>
       </c>
-      <c r="I14" s="10" t="s">
-        <v>194</v>
-      </c>
-      <c r="J14" s="10" t="s">
-        <v>227</v>
-      </c>
-      <c r="K14" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="L14" s="8" t="s">
+      <c r="I14" s="8" t="s">
+        <v>191</v>
+      </c>
+      <c r="J14" s="8" t="s">
+        <v>223</v>
+      </c>
+      <c r="K14" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="L14" s="6" t="s">
         <v>99</v>
       </c>
-      <c r="M14" s="8"/>
-      <c r="N14" s="7"/>
-      <c r="O14" s="8"/>
-      <c r="P14" s="5">
+      <c r="M14" s="6">
+        <v>1</v>
+      </c>
+      <c r="N14" s="5">
+        <f t="shared" si="5"/>
+        <v>46093</v>
+      </c>
+      <c r="O14" s="3">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="P14" s="3">
         <f t="shared" si="2"/>
-        <v>-1</v>
-      </c>
-      <c r="Q14" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="Q14" s="6" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="15" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A15" s="4" t="s">
+      <c r="A15" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="B15" s="5">
-        <v>1</v>
-      </c>
-      <c r="C15" s="6">
+      <c r="B15" s="3">
+        <v>1</v>
+      </c>
+      <c r="C15" s="4">
         <v>0.44</v>
       </c>
-      <c r="D15" s="6">
+      <c r="D15" s="4">
         <f t="shared" si="0"/>
         <v>0.44</v>
       </c>
-      <c r="E15" s="6">
+      <c r="E15" s="4">
         <f t="shared" si="3"/>
         <v>0.44</v>
       </c>
-      <c r="F15" s="6">
+      <c r="F15" s="4">
         <f t="shared" si="1"/>
         <v>0.44</v>
       </c>
-      <c r="G15" s="8" t="s">
+      <c r="G15" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="H15" s="8" t="s">
+      <c r="H15" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="I15" s="10" t="s">
-        <v>193</v>
-      </c>
-      <c r="J15" s="10" t="s">
+      <c r="I15" s="8" t="s">
+        <v>190</v>
+      </c>
+      <c r="J15" s="8" t="s">
         <v>85</v>
       </c>
-      <c r="K15" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="L15" s="8" t="s">
+      <c r="K15" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="L15" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="M15" s="8"/>
-      <c r="N15" s="7"/>
-      <c r="O15" s="8"/>
-      <c r="P15" s="5">
+      <c r="M15" s="6">
+        <v>1</v>
+      </c>
+      <c r="N15" s="5">
+        <f t="shared" si="5"/>
+        <v>46093</v>
+      </c>
+      <c r="O15" s="3">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="P15" s="3">
         <f t="shared" si="2"/>
-        <v>-1</v>
-      </c>
-      <c r="Q15" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="Q15" s="6" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="16" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A16" s="4" t="s">
+      <c r="A16" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="B16" s="5">
-        <v>1</v>
-      </c>
-      <c r="C16" s="6">
+      <c r="B16" s="3">
+        <v>1</v>
+      </c>
+      <c r="C16" s="4">
         <v>0.24</v>
       </c>
-      <c r="D16" s="6">
+      <c r="D16" s="4">
         <f t="shared" si="0"/>
         <v>0.24</v>
       </c>
-      <c r="E16" s="6">
+      <c r="E16" s="4">
         <f t="shared" si="3"/>
         <v>0.24</v>
       </c>
-      <c r="F16" s="6">
+      <c r="F16" s="4">
         <f t="shared" si="1"/>
         <v>0.24</v>
       </c>
-      <c r="G16" s="8" t="s">
+      <c r="G16" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="H16" s="8" t="s">
+      <c r="H16" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="I16" s="10" t="s">
-        <v>195</v>
-      </c>
-      <c r="J16" s="10" t="s">
+      <c r="I16" s="8" t="s">
+        <v>192</v>
+      </c>
+      <c r="J16" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="K16" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="L16" s="8" t="s">
+      <c r="K16" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="L16" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="M16" s="8"/>
-      <c r="N16" s="7"/>
-      <c r="O16" s="8"/>
-      <c r="P16" s="5">
+      <c r="M16" s="6">
+        <v>1</v>
+      </c>
+      <c r="N16" s="5">
+        <f t="shared" si="5"/>
+        <v>46093</v>
+      </c>
+      <c r="O16" s="3">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="P16" s="3">
         <f t="shared" si="2"/>
-        <v>-1</v>
-      </c>
-      <c r="Q16" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="Q16" s="6" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="17" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A17" s="4" t="s">
-        <v>172</v>
-      </c>
-      <c r="B17" s="5">
-        <v>1</v>
-      </c>
-      <c r="C17" s="6">
+      <c r="A17" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="B17" s="3">
+        <v>1</v>
+      </c>
+      <c r="C17" s="4">
         <v>0.53</v>
       </c>
-      <c r="D17" s="6">
+      <c r="D17" s="4">
         <f t="shared" si="0"/>
         <v>0.53</v>
       </c>
-      <c r="E17" s="6">
+      <c r="E17" s="4">
         <f t="shared" si="3"/>
         <v>0.53</v>
       </c>
-      <c r="F17" s="6">
+      <c r="F17" s="4">
         <f t="shared" si="1"/>
         <v>0.53</v>
       </c>
-      <c r="G17" s="8" t="s">
+      <c r="G17" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="H17" s="6" t="s">
+        <v>171</v>
+      </c>
+      <c r="I17" s="8" t="s">
+        <v>193</v>
+      </c>
+      <c r="J17" s="8" t="s">
+        <v>224</v>
+      </c>
+      <c r="K17" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="L17" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="M17" s="6">
+        <v>1</v>
+      </c>
+      <c r="N17" s="5">
+        <f t="shared" si="5"/>
+        <v>46093</v>
+      </c>
+      <c r="O17" s="3">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="P17" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="Q17" s="6" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="18" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A18" s="2" t="s">
         <v>173</v>
       </c>
-      <c r="H17" s="8" t="s">
-        <v>174</v>
-      </c>
-      <c r="I17" s="10" t="s">
-        <v>196</v>
-      </c>
-      <c r="J17" s="10" t="s">
-        <v>228</v>
-      </c>
-      <c r="K17" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="L17" s="8" t="s">
-        <v>175</v>
-      </c>
-      <c r="M17" s="8"/>
-      <c r="N17" s="7"/>
-      <c r="O17" s="8"/>
-      <c r="P17" s="5">
-        <f t="shared" si="2"/>
-        <v>-1</v>
-      </c>
-      <c r="Q17" s="8" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="18" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A18" s="4" t="s">
-        <v>176</v>
-      </c>
-      <c r="B18" s="5">
-        <v>1</v>
-      </c>
-      <c r="C18" s="6">
+      <c r="B18" s="3">
+        <v>1</v>
+      </c>
+      <c r="C18" s="4">
         <v>1.39</v>
       </c>
-      <c r="D18" s="6">
+      <c r="D18" s="4">
         <f t="shared" si="0"/>
         <v>1.39</v>
       </c>
-      <c r="E18" s="6">
+      <c r="E18" s="4">
         <f t="shared" si="3"/>
         <v>1.39</v>
       </c>
-      <c r="F18" s="6">
+      <c r="F18" s="4">
         <f t="shared" si="1"/>
         <v>1.39</v>
       </c>
-      <c r="G18" s="8" t="s">
-        <v>173</v>
-      </c>
-      <c r="H18" s="8" t="s">
-        <v>177</v>
-      </c>
-      <c r="I18" s="10" t="s">
-        <v>197</v>
-      </c>
-      <c r="J18" s="10" t="s">
-        <v>229</v>
-      </c>
-      <c r="K18" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="L18" s="8" t="s">
-        <v>178</v>
-      </c>
-      <c r="M18" s="8"/>
-      <c r="N18" s="7"/>
-      <c r="O18" s="8"/>
-      <c r="P18" s="5">
+      <c r="G18" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="H18" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="I18" s="8" t="s">
+        <v>194</v>
+      </c>
+      <c r="J18" s="8" t="s">
+        <v>225</v>
+      </c>
+      <c r="K18" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="L18" s="6" t="s">
+        <v>175</v>
+      </c>
+      <c r="M18" s="6">
+        <v>1</v>
+      </c>
+      <c r="N18" s="5">
+        <f t="shared" si="5"/>
+        <v>46093</v>
+      </c>
+      <c r="O18" s="3">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="P18" s="3">
         <f t="shared" si="2"/>
-        <v>-1</v>
-      </c>
-      <c r="Q18" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="Q18" s="6" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="19" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A19" s="4" t="s">
+      <c r="A19" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="B19" s="5">
-        <v>1</v>
-      </c>
-      <c r="C19" s="6">
+      <c r="B19" s="3">
+        <v>1</v>
+      </c>
+      <c r="C19" s="4">
         <v>0.52</v>
       </c>
-      <c r="D19" s="6">
+      <c r="D19" s="4">
         <f t="shared" si="0"/>
         <v>0.52</v>
       </c>
-      <c r="E19" s="6">
+      <c r="E19" s="4">
         <f t="shared" si="3"/>
         <v>0.52</v>
       </c>
-      <c r="F19" s="6">
+      <c r="F19" s="4">
         <f t="shared" si="1"/>
         <v>0.52</v>
       </c>
-      <c r="G19" s="8" t="s">
+      <c r="G19" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="H19" s="8" t="s">
+      <c r="H19" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="I19" s="11" t="s">
-        <v>198</v>
-      </c>
-      <c r="J19" s="10" t="s">
-        <v>230</v>
-      </c>
-      <c r="K19" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="L19" s="8" t="s">
+      <c r="I19" s="9" t="s">
+        <v>195</v>
+      </c>
+      <c r="J19" s="8" t="s">
+        <v>226</v>
+      </c>
+      <c r="K19" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="L19" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="M19" s="8"/>
-      <c r="N19" s="7"/>
-      <c r="O19" s="8"/>
-      <c r="P19" s="5">
+      <c r="M19" s="6">
+        <v>1</v>
+      </c>
+      <c r="N19" s="5">
+        <f t="shared" si="5"/>
+        <v>46093</v>
+      </c>
+      <c r="O19" s="3">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="P19" s="3">
         <f t="shared" si="2"/>
-        <v>-1</v>
-      </c>
-      <c r="Q19" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="Q19" s="6" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="20" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A20" s="4" t="s">
-        <v>179</v>
-      </c>
-      <c r="B20" s="5">
-        <v>1</v>
-      </c>
-      <c r="C20" s="6">
+      <c r="A20" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="B20" s="3">
+        <v>1</v>
+      </c>
+      <c r="C20" s="4">
         <v>0.51</v>
       </c>
-      <c r="D20" s="6">
-        <f t="shared" ref="D20" si="4">B20*C20</f>
+      <c r="D20" s="4">
+        <f t="shared" ref="D20" si="6">B20*C20</f>
         <v>0.51</v>
       </c>
-      <c r="E20" s="6">
-        <f t="shared" ref="E20" si="5">C20</f>
+      <c r="E20" s="4">
+        <f t="shared" ref="E20" si="7">C20</f>
         <v>0.51</v>
       </c>
-      <c r="F20" s="6">
-        <f t="shared" ref="F20" si="6">B20*E20</f>
+      <c r="F20" s="4">
+        <f t="shared" ref="F20" si="8">B20*E20</f>
         <v>0.51</v>
       </c>
-      <c r="G20" s="8" t="s">
-        <v>173</v>
-      </c>
-      <c r="H20" s="8" t="s">
-        <v>180</v>
-      </c>
-      <c r="I20" s="10" t="s">
-        <v>199</v>
-      </c>
-      <c r="J20" s="10" t="s">
-        <v>231</v>
-      </c>
-      <c r="K20" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="L20" s="8" t="s">
-        <v>181</v>
-      </c>
-      <c r="M20" s="8"/>
-      <c r="N20" s="7"/>
-      <c r="O20" s="8"/>
-      <c r="P20" s="5">
+      <c r="G20" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="H20" s="6" t="s">
+        <v>177</v>
+      </c>
+      <c r="I20" s="8" t="s">
+        <v>196</v>
+      </c>
+      <c r="J20" s="8" t="s">
+        <v>227</v>
+      </c>
+      <c r="K20" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="L20" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="M20" s="6">
+        <v>1</v>
+      </c>
+      <c r="N20" s="5">
+        <f t="shared" si="5"/>
+        <v>46093</v>
+      </c>
+      <c r="O20" s="3">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="P20" s="3">
         <f t="shared" si="2"/>
-        <v>-1</v>
-      </c>
-      <c r="Q20" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="Q20" s="6" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="21" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A21" s="4" t="s">
+      <c r="A21" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="B21" s="5">
-        <v>1</v>
-      </c>
-      <c r="C21" s="6">
+      <c r="B21" s="3">
+        <v>1</v>
+      </c>
+      <c r="C21" s="4">
         <v>0.52</v>
       </c>
-      <c r="D21" s="6">
+      <c r="D21" s="4">
         <f t="shared" si="0"/>
         <v>0.52</v>
       </c>
-      <c r="E21" s="6">
+      <c r="E21" s="4">
         <f t="shared" si="3"/>
         <v>0.52</v>
       </c>
-      <c r="F21" s="6">
+      <c r="F21" s="4">
         <f t="shared" si="1"/>
         <v>0.52</v>
       </c>
-      <c r="G21" s="8" t="s">
+      <c r="G21" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="H21" s="8" t="s">
+      <c r="H21" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="I21" s="10" t="s">
-        <v>200</v>
-      </c>
-      <c r="J21" s="10" t="s">
-        <v>230</v>
-      </c>
-      <c r="K21" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="L21" s="8" t="s">
+      <c r="I21" s="8" t="s">
+        <v>197</v>
+      </c>
+      <c r="J21" s="8" t="s">
+        <v>226</v>
+      </c>
+      <c r="K21" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="L21" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="M21" s="8"/>
-      <c r="N21" s="7"/>
-      <c r="O21" s="8"/>
-      <c r="P21" s="5">
+      <c r="M21" s="6">
+        <v>1</v>
+      </c>
+      <c r="N21" s="5">
+        <f t="shared" si="5"/>
+        <v>46093</v>
+      </c>
+      <c r="O21" s="3">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="P21" s="3">
         <f t="shared" si="2"/>
-        <v>-1</v>
-      </c>
-      <c r="Q21" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="Q21" s="6" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="22" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A22" s="4" t="s">
-        <v>152</v>
-      </c>
-      <c r="B22" s="5">
-        <v>5</v>
-      </c>
-      <c r="C22" s="6">
+      <c r="A22" s="2" t="s">
+        <v>264</v>
+      </c>
+      <c r="B22" s="3">
+        <v>1</v>
+      </c>
+      <c r="C22" s="4">
+        <v>10</v>
+      </c>
+      <c r="D22" s="4">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="E22" s="4">
+        <f t="shared" ref="E22:E23" si="9">C22</f>
+        <v>10</v>
+      </c>
+      <c r="F22" s="4">
+        <f t="shared" ref="F22:F23" si="10">B22*E22</f>
+        <v>10</v>
+      </c>
+      <c r="G22" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="H22" s="6" t="s">
+        <v>265</v>
+      </c>
+      <c r="I22" s="8" t="s">
+        <v>266</v>
+      </c>
+      <c r="J22" s="8" t="s">
+        <v>268</v>
+      </c>
+      <c r="K22" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="L22" s="6" t="s">
+        <v>267</v>
+      </c>
+      <c r="M22" s="6">
+        <v>0</v>
+      </c>
+      <c r="N22" s="5">
+        <f t="shared" si="5"/>
+        <v>46093</v>
+      </c>
+      <c r="O22" s="3">
+        <v>1</v>
+      </c>
+      <c r="P22" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="Q22" s="6" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="23" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A23" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="B23" s="3">
+        <v>1</v>
+      </c>
+      <c r="C23" s="4">
+        <v>0.1</v>
+      </c>
+      <c r="D23" s="4">
+        <f t="shared" si="0"/>
+        <v>0.1</v>
+      </c>
+      <c r="E23" s="4">
+        <f t="shared" si="9"/>
+        <v>0.1</v>
+      </c>
+      <c r="F23" s="4">
+        <f t="shared" si="10"/>
+        <v>0.1</v>
+      </c>
+      <c r="G23" s="6" t="s">
+        <v>258</v>
+      </c>
+      <c r="H23" s="6" t="s">
+        <v>257</v>
+      </c>
+      <c r="I23" s="8" t="s">
+        <v>259</v>
+      </c>
+      <c r="J23" s="8" t="s">
+        <v>260</v>
+      </c>
+      <c r="K23" s="13" t="s">
+        <v>60</v>
+      </c>
+      <c r="L23" s="6" t="s">
+        <v>261</v>
+      </c>
+      <c r="M23" s="6">
+        <v>0</v>
+      </c>
+      <c r="N23" s="5">
+        <f t="shared" si="5"/>
+        <v>46093</v>
+      </c>
+      <c r="O23" s="3">
+        <v>1</v>
+      </c>
+      <c r="P23" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="Q23" s="6" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="24" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A24" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="B24" s="3">
+        <v>3</v>
+      </c>
+      <c r="C24" s="4">
         <v>0.4</v>
       </c>
-      <c r="D22" s="6">
+      <c r="D24" s="4">
         <f t="shared" si="0"/>
-        <v>2</v>
-      </c>
-      <c r="E22" s="6">
+        <v>1.2000000000000002</v>
+      </c>
+      <c r="E24" s="4">
         <f t="shared" si="3"/>
         <v>0.4</v>
       </c>
-      <c r="F22" s="6">
+      <c r="F24" s="4">
         <f t="shared" si="1"/>
-        <v>2</v>
-      </c>
-      <c r="G22" s="8" t="s">
+        <v>1.2000000000000002</v>
+      </c>
+      <c r="G24" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="H24" s="6" t="s">
+        <v>151</v>
+      </c>
+      <c r="I24" s="8" t="s">
+        <v>198</v>
+      </c>
+      <c r="J24" s="8" t="s">
+        <v>228</v>
+      </c>
+      <c r="K24" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="L24" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="M24" s="6">
+        <v>7</v>
+      </c>
+      <c r="N24" s="5">
+        <f t="shared" si="5"/>
+        <v>46093</v>
+      </c>
+      <c r="O24" s="3">
+        <f t="shared" si="4"/>
+        <v>7</v>
+      </c>
+      <c r="P24" s="3">
+        <f t="shared" si="2"/>
+        <v>4</v>
+      </c>
+      <c r="Q24" s="6" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="25" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A25" s="2" t="s">
         <v>153</v>
       </c>
-      <c r="H22" s="8" t="s">
-        <v>154</v>
-      </c>
-      <c r="I22" s="10" t="s">
-        <v>201</v>
-      </c>
-      <c r="J22" s="10" t="s">
-        <v>232</v>
-      </c>
-      <c r="K22" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="L22" s="8" t="s">
-        <v>155</v>
-      </c>
-      <c r="M22" s="8"/>
-      <c r="N22" s="7"/>
-      <c r="O22" s="8"/>
-      <c r="P22" s="5">
-        <f t="shared" si="2"/>
-        <v>-5</v>
-      </c>
-      <c r="Q22" s="8" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="23" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A23" s="4" t="s">
-        <v>156</v>
-      </c>
-      <c r="B23" s="5">
-        <v>1</v>
-      </c>
-      <c r="C23" s="6">
+      <c r="B25" s="3">
+        <v>1</v>
+      </c>
+      <c r="C25" s="4">
         <v>0.1</v>
       </c>
-      <c r="D23" s="6">
+      <c r="D25" s="4">
         <f t="shared" si="0"/>
         <v>0.1</v>
       </c>
-      <c r="E23" s="6">
+      <c r="E25" s="4">
         <f t="shared" si="3"/>
         <v>0.1</v>
       </c>
-      <c r="F23" s="6">
+      <c r="F25" s="4">
         <f t="shared" si="1"/>
         <v>0.1</v>
       </c>
-      <c r="G23" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="H23" s="8" t="s">
-        <v>158</v>
-      </c>
-      <c r="I23" s="10" t="s">
-        <v>202</v>
-      </c>
-      <c r="J23" s="10" t="s">
-        <v>233</v>
-      </c>
-      <c r="K23" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="L23" s="8" t="s">
-        <v>159</v>
-      </c>
-      <c r="M23" s="8"/>
-      <c r="N23" s="7"/>
-      <c r="O23" s="8"/>
-      <c r="P23" s="5">
+      <c r="G25" s="6" t="s">
+        <v>154</v>
+      </c>
+      <c r="H25" s="6" t="s">
+        <v>155</v>
+      </c>
+      <c r="I25" s="8" t="s">
+        <v>199</v>
+      </c>
+      <c r="J25" s="8" t="s">
+        <v>229</v>
+      </c>
+      <c r="K25" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="L25" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="M25" s="6">
+        <v>1</v>
+      </c>
+      <c r="N25" s="5">
+        <f t="shared" si="5"/>
+        <v>46093</v>
+      </c>
+      <c r="O25" s="3">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="P25" s="3">
         <f t="shared" si="2"/>
-        <v>-1</v>
-      </c>
-      <c r="Q23" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="Q25" s="6" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="24" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A24" s="4" t="s">
-        <v>150</v>
-      </c>
-      <c r="B24" s="5">
-        <v>1</v>
-      </c>
-      <c r="C24" s="6">
+    <row r="26" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A26" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="B26" s="3">
+        <v>1</v>
+      </c>
+      <c r="C26" s="4">
         <v>0.63</v>
       </c>
-      <c r="D24" s="6">
+      <c r="D26" s="4">
         <f t="shared" si="0"/>
         <v>0.63</v>
       </c>
-      <c r="E24" s="6">
+      <c r="E26" s="4">
         <f t="shared" si="3"/>
         <v>0.63</v>
       </c>
-      <c r="F24" s="6">
+      <c r="F26" s="4">
         <f t="shared" si="1"/>
         <v>0.63</v>
       </c>
-      <c r="G24" s="8" t="s">
+      <c r="G26" s="6" t="s">
+        <v>145</v>
+      </c>
+      <c r="H26" s="6">
+        <v>34.312399999999997</v>
+      </c>
+      <c r="I26" s="8" t="s">
+        <v>200</v>
+      </c>
+      <c r="J26" s="8" t="s">
+        <v>230</v>
+      </c>
+      <c r="K26" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="L26" s="6" t="s">
         <v>148</v>
       </c>
-      <c r="H24" s="8">
-        <v>34.312399999999997</v>
-      </c>
-      <c r="I24" s="10" t="s">
-        <v>203</v>
-      </c>
-      <c r="J24" s="10" t="s">
-        <v>234</v>
-      </c>
-      <c r="K24" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="L24" s="8" t="s">
-        <v>151</v>
-      </c>
-      <c r="M24" s="8"/>
-      <c r="N24" s="7"/>
-      <c r="O24" s="8"/>
-      <c r="P24" s="5">
+      <c r="M26" s="6">
+        <v>0</v>
+      </c>
+      <c r="N26" s="5">
+        <f t="shared" si="5"/>
+        <v>46093</v>
+      </c>
+      <c r="O26" s="3">
+        <v>1</v>
+      </c>
+      <c r="P26" s="3">
         <f t="shared" si="2"/>
-        <v>-1</v>
-      </c>
-      <c r="Q24" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="Q26" s="6" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="25" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A25" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="B25" s="5">
-        <v>1</v>
-      </c>
-      <c r="C25" s="6">
+    <row r="27" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A27" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="B27" s="3">
+        <v>1</v>
+      </c>
+      <c r="C27" s="4">
         <v>0.63</v>
       </c>
-      <c r="D25" s="6">
+      <c r="D27" s="4">
         <f t="shared" si="0"/>
         <v>0.63</v>
       </c>
-      <c r="E25" s="6">
+      <c r="E27" s="4">
         <f t="shared" si="3"/>
         <v>0.63</v>
       </c>
-      <c r="F25" s="6">
+      <c r="F27" s="4">
         <f t="shared" si="1"/>
         <v>0.63</v>
       </c>
-      <c r="G25" s="8" t="s">
-        <v>148</v>
-      </c>
-      <c r="H25" s="8">
+      <c r="G27" s="6" t="s">
+        <v>145</v>
+      </c>
+      <c r="H27" s="6">
         <v>34.3123</v>
       </c>
-      <c r="I25" s="10" t="s">
-        <v>204</v>
-      </c>
-      <c r="J25" s="10" t="s">
-        <v>235</v>
-      </c>
-      <c r="K25" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="L25" s="8" t="s">
-        <v>149</v>
-      </c>
-      <c r="M25" s="8"/>
-      <c r="N25" s="7"/>
-      <c r="O25" s="8"/>
-      <c r="P25" s="5">
+      <c r="I27" s="8" t="s">
+        <v>201</v>
+      </c>
+      <c r="J27" s="8" t="s">
+        <v>231</v>
+      </c>
+      <c r="K27" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="L27" s="6" t="s">
+        <v>146</v>
+      </c>
+      <c r="M27" s="6">
+        <v>5</v>
+      </c>
+      <c r="N27" s="5">
+        <f t="shared" si="5"/>
+        <v>46093</v>
+      </c>
+      <c r="O27" s="3">
+        <f t="shared" si="4"/>
+        <v>5</v>
+      </c>
+      <c r="P27" s="3">
         <f t="shared" si="2"/>
-        <v>-1</v>
-      </c>
-      <c r="Q25" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="Q27" s="6" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="26" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A26" s="4" t="s">
+    <row r="28" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A28" s="14" t="s">
         <v>140</v>
       </c>
-      <c r="B26" s="5">
-        <v>1</v>
-      </c>
-      <c r="C26" s="6">
-        <v>1.03</v>
-      </c>
-      <c r="D26" s="6">
+      <c r="B28" s="3">
+        <v>1</v>
+      </c>
+      <c r="C28" s="4">
+        <v>0.19</v>
+      </c>
+      <c r="D28" s="4">
         <f t="shared" si="0"/>
-        <v>1.03</v>
-      </c>
-      <c r="E26" s="6">
+        <v>0.19</v>
+      </c>
+      <c r="E28" s="4">
         <f t="shared" si="3"/>
-        <v>1.03</v>
-      </c>
-      <c r="F26" s="6">
+        <v>0.19</v>
+      </c>
+      <c r="F28" s="4">
         <f t="shared" si="1"/>
-        <v>1.03</v>
-      </c>
-      <c r="G26" s="8" t="s">
+        <v>0.19</v>
+      </c>
+      <c r="G28" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="H28" s="6" t="s">
+        <v>269</v>
+      </c>
+      <c r="I28" s="8" t="s">
+        <v>270</v>
+      </c>
+      <c r="J28" s="8" t="s">
+        <v>271</v>
+      </c>
+      <c r="K28" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="L28" s="6" t="s">
+        <v>272</v>
+      </c>
+      <c r="M28" s="6">
+        <v>0</v>
+      </c>
+      <c r="N28" s="5">
+        <f t="shared" si="5"/>
+        <v>46093</v>
+      </c>
+      <c r="O28" s="3">
+        <v>1</v>
+      </c>
+      <c r="P28" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="Q28" s="6" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="29" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A29" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="H26" s="8" t="s">
-        <v>142</v>
-      </c>
-      <c r="I26" s="10" t="s">
-        <v>205</v>
-      </c>
-      <c r="J26" s="10" t="s">
-        <v>236</v>
-      </c>
-      <c r="K26" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="L26" s="8" t="s">
-        <v>143</v>
-      </c>
-      <c r="M26" s="8"/>
-      <c r="N26" s="7"/>
-      <c r="O26" s="8"/>
-      <c r="P26" s="5">
-        <f t="shared" si="2"/>
-        <v>-1</v>
-      </c>
-      <c r="Q26" s="8" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="27" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A27" s="4" t="s">
-        <v>144</v>
-      </c>
-      <c r="B27" s="5">
-        <v>1</v>
-      </c>
-      <c r="C27" s="6">
+      <c r="B29" s="3">
+        <v>1</v>
+      </c>
+      <c r="C29" s="4">
         <v>1.06</v>
       </c>
-      <c r="D27" s="6">
+      <c r="D29" s="4">
         <f t="shared" si="0"/>
         <v>1.06</v>
       </c>
-      <c r="E27" s="6">
+      <c r="E29" s="4">
         <f t="shared" si="3"/>
         <v>1.06</v>
       </c>
-      <c r="F27" s="6">
+      <c r="F29" s="4">
         <f t="shared" si="1"/>
         <v>1.06</v>
       </c>
-      <c r="G27" s="8" t="s">
+      <c r="G29" s="6" t="s">
         <v>101</v>
       </c>
-      <c r="H27" s="8" t="s">
-        <v>145</v>
-      </c>
-      <c r="I27" s="10" t="s">
-        <v>206</v>
-      </c>
-      <c r="J27" s="10" t="s">
-        <v>237</v>
-      </c>
-      <c r="K27" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="L27" s="8" t="s">
-        <v>146</v>
-      </c>
-      <c r="M27" s="8"/>
-      <c r="N27" s="7"/>
-      <c r="O27" s="8"/>
-      <c r="P27" s="5">
+      <c r="H29" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="I29" s="8" t="s">
+        <v>202</v>
+      </c>
+      <c r="J29" s="8" t="s">
+        <v>232</v>
+      </c>
+      <c r="K29" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="L29" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="M29" s="6">
+        <v>1</v>
+      </c>
+      <c r="N29" s="5">
+        <f t="shared" si="5"/>
+        <v>46093</v>
+      </c>
+      <c r="O29" s="3">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="P29" s="3">
         <f t="shared" si="2"/>
-        <v>-1</v>
-      </c>
-      <c r="Q27" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="Q29" s="6" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="28" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A28" s="4" t="s">
+    <row r="30" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A30" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="B28" s="5">
+      <c r="B30" s="3">
         <v>2</v>
       </c>
-      <c r="C28" s="6">
+      <c r="C30" s="4">
         <v>5.95</v>
       </c>
-      <c r="D28" s="6">
+      <c r="D30" s="4">
         <f t="shared" si="0"/>
         <v>11.9</v>
       </c>
-      <c r="E28" s="6">
+      <c r="E30" s="4">
         <f t="shared" si="3"/>
         <v>5.95</v>
       </c>
-      <c r="F28" s="6">
+      <c r="F30" s="4">
         <f t="shared" si="1"/>
         <v>11.9</v>
       </c>
-      <c r="G28" s="8" t="s">
+      <c r="G30" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="H28" s="8">
+      <c r="H30" s="6">
         <v>4326</v>
       </c>
-      <c r="I28" s="10" t="s">
-        <v>207</v>
-      </c>
-      <c r="J28" s="10" t="s">
-        <v>238</v>
-      </c>
-      <c r="K28" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="L28" s="8" t="s">
+      <c r="I30" s="8" t="s">
+        <v>203</v>
+      </c>
+      <c r="J30" s="8" t="s">
+        <v>233</v>
+      </c>
+      <c r="K30" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="L30" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="M28" s="8"/>
-      <c r="N28" s="7"/>
-      <c r="O28" s="8"/>
-      <c r="P28" s="5">
+      <c r="M30" s="6">
+        <v>3</v>
+      </c>
+      <c r="N30" s="5">
+        <f t="shared" si="5"/>
+        <v>46093</v>
+      </c>
+      <c r="O30" s="3">
+        <f t="shared" si="4"/>
+        <v>3</v>
+      </c>
+      <c r="P30" s="3">
         <f t="shared" si="2"/>
-        <v>-2</v>
-      </c>
-      <c r="Q28" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="Q30" s="6" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="29" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A29" s="4" t="s">
-        <v>164</v>
-      </c>
-      <c r="B29" s="5">
+    <row r="31" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A31" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="B31" s="3">
         <v>3</v>
       </c>
-      <c r="C29" s="6">
+      <c r="C31" s="4">
         <v>3.71</v>
       </c>
-      <c r="D29" s="6">
+      <c r="D31" s="4">
         <f t="shared" si="0"/>
         <v>11.129999999999999</v>
       </c>
-      <c r="E29" s="6">
+      <c r="E31" s="4">
         <f t="shared" si="3"/>
         <v>3.71</v>
       </c>
-      <c r="F29" s="6">
+      <c r="F31" s="4">
         <f t="shared" si="1"/>
         <v>11.129999999999999</v>
       </c>
-      <c r="G29" s="8" t="s">
-        <v>165</v>
-      </c>
-      <c r="H29" s="8" t="s">
-        <v>166</v>
-      </c>
-      <c r="I29" s="10" t="s">
-        <v>208</v>
-      </c>
-      <c r="J29" s="10" t="s">
-        <v>239</v>
-      </c>
-      <c r="K29" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="L29" s="8" t="s">
-        <v>167</v>
-      </c>
-      <c r="M29" s="8"/>
-      <c r="N29" s="7"/>
-      <c r="O29" s="8"/>
-      <c r="P29" s="5">
+      <c r="G31" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="H31" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="I31" s="8" t="s">
+        <v>204</v>
+      </c>
+      <c r="J31" s="8" t="s">
+        <v>234</v>
+      </c>
+      <c r="K31" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="L31" s="6" t="s">
+        <v>164</v>
+      </c>
+      <c r="M31" s="6">
+        <v>3</v>
+      </c>
+      <c r="N31" s="5">
+        <f t="shared" si="5"/>
+        <v>46093</v>
+      </c>
+      <c r="O31" s="3">
+        <f t="shared" si="4"/>
+        <v>3</v>
+      </c>
+      <c r="P31" s="3">
         <f t="shared" si="2"/>
-        <v>-3</v>
-      </c>
-      <c r="Q29" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="Q31" s="6" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="30" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A30" s="4" t="s">
+    <row r="32" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A32" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B30" s="5">
+      <c r="B32" s="3">
         <v>2</v>
       </c>
-      <c r="C30" s="6">
+      <c r="C32" s="4">
         <v>1.48</v>
       </c>
-      <c r="D30" s="6">
+      <c r="D32" s="4">
         <f t="shared" si="0"/>
         <v>2.96</v>
       </c>
-      <c r="E30" s="6">
+      <c r="E32" s="4">
         <f t="shared" si="3"/>
         <v>1.48</v>
       </c>
-      <c r="F30" s="6">
+      <c r="F32" s="4">
         <f t="shared" si="1"/>
         <v>2.96</v>
       </c>
-      <c r="G30" s="8" t="s">
-        <v>249</v>
-      </c>
-      <c r="H30" s="8">
+      <c r="G32" s="6" t="s">
+        <v>244</v>
+      </c>
+      <c r="H32" s="6">
         <v>702460801</v>
       </c>
-      <c r="I30" s="10" t="s">
-        <v>250</v>
-      </c>
-      <c r="J30" s="10" t="s">
-        <v>256</v>
-      </c>
-      <c r="K30" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="L30" s="8" t="s">
+      <c r="I32" s="8" t="s">
+        <v>245</v>
+      </c>
+      <c r="J32" s="8" t="s">
         <v>251</v>
       </c>
-      <c r="M30" s="8"/>
-      <c r="N30" s="7"/>
-      <c r="O30" s="8"/>
-      <c r="P30" s="5">
+      <c r="K32" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="L32" s="6" t="s">
+        <v>246</v>
+      </c>
+      <c r="M32" s="6">
+        <v>0</v>
+      </c>
+      <c r="N32" s="5">
+        <f t="shared" si="5"/>
+        <v>46093</v>
+      </c>
+      <c r="O32" s="3">
+        <v>2</v>
+      </c>
+      <c r="P32" s="3">
         <f t="shared" si="2"/>
-        <v>-2</v>
-      </c>
-      <c r="Q30" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="Q32" s="6" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="31" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A31" s="4" t="s">
+    <row r="33" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A33" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B31" s="5">
+      <c r="B33" s="3">
         <v>2</v>
       </c>
-      <c r="C31" s="6">
+      <c r="C33" s="4">
         <v>5</v>
       </c>
-      <c r="D31" s="6">
+      <c r="D33" s="4">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="E31" s="6">
+      <c r="E33" s="4">
         <f t="shared" si="3"/>
         <v>5</v>
       </c>
-      <c r="F31" s="6">
+      <c r="F33" s="4">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="G31" s="8" t="s">
+      <c r="G33" s="6" t="s">
+        <v>247</v>
+      </c>
+      <c r="H33" s="6" t="s">
+        <v>248</v>
+      </c>
+      <c r="I33" s="8" t="s">
+        <v>250</v>
+      </c>
+      <c r="J33" s="8" t="s">
+        <v>249</v>
+      </c>
+      <c r="K33" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="L33" s="6" t="s">
         <v>252</v>
       </c>
-      <c r="H31" s="8" t="s">
-        <v>253</v>
-      </c>
-      <c r="I31" s="10" t="s">
-        <v>255</v>
-      </c>
-      <c r="J31" s="10" t="s">
-        <v>254</v>
-      </c>
-      <c r="K31" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="L31" s="8" t="s">
-        <v>257</v>
-      </c>
-      <c r="M31" s="8"/>
-      <c r="N31" s="8"/>
-      <c r="O31" s="8"/>
-      <c r="P31" s="8">
-        <f t="shared" ref="H31:Q31" si="7">P30</f>
-        <v>-2</v>
-      </c>
-      <c r="Q31" s="8" t="str">
-        <f t="shared" si="7"/>
+      <c r="M33" s="6">
+        <v>0</v>
+      </c>
+      <c r="N33" s="5">
+        <f t="shared" si="5"/>
+        <v>46093</v>
+      </c>
+      <c r="O33" s="3">
+        <v>2</v>
+      </c>
+      <c r="P33" s="6">
+        <f t="shared" ref="P33:Q33" si="11">P32</f>
+        <v>0</v>
+      </c>
+      <c r="Q33" s="6" t="str">
+        <f t="shared" si="11"/>
         <v>J3, J4</v>
       </c>
     </row>
-    <row r="32" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A32" s="4" t="s">
+    <row r="34" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A34" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="B32" s="5">
-        <v>1</v>
-      </c>
-      <c r="C32" s="6">
+      <c r="B34" s="3">
+        <v>1</v>
+      </c>
+      <c r="C34" s="4">
         <v>0.71</v>
       </c>
-      <c r="D32" s="6">
+      <c r="D34" s="4">
         <f t="shared" si="0"/>
         <v>0.71</v>
       </c>
-      <c r="E32" s="6">
+      <c r="E34" s="4">
         <f t="shared" si="3"/>
         <v>0.71</v>
       </c>
-      <c r="F32" s="6">
+      <c r="F34" s="4">
         <f t="shared" si="1"/>
         <v>0.71</v>
       </c>
-      <c r="G32" s="8" t="s">
+      <c r="G34" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="H32" s="8" t="s">
+      <c r="H34" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="I32" s="10" t="s">
-        <v>209</v>
-      </c>
-      <c r="J32" s="10" t="s">
-        <v>240</v>
-      </c>
-      <c r="K32" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="L32" s="8" t="s">
+      <c r="I34" s="8" t="s">
+        <v>205</v>
+      </c>
+      <c r="J34" s="8" t="s">
+        <v>235</v>
+      </c>
+      <c r="K34" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="L34" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="M32" s="8"/>
-      <c r="N32" s="7"/>
-      <c r="O32" s="8"/>
-      <c r="P32" s="5">
+      <c r="M34" s="6">
+        <v>1</v>
+      </c>
+      <c r="N34" s="5">
+        <f t="shared" si="5"/>
+        <v>46093</v>
+      </c>
+      <c r="O34" s="3">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="P34" s="3">
         <f t="shared" si="2"/>
-        <v>-1</v>
-      </c>
-      <c r="Q32" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="Q34" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="33" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A33" s="4" t="s">
+    <row r="35" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A35" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="B33" s="5">
-        <v>1</v>
-      </c>
-      <c r="C33" s="6">
+      <c r="B35" s="3">
+        <v>1</v>
+      </c>
+      <c r="C35" s="4">
         <v>0.77</v>
       </c>
-      <c r="D33" s="6">
+      <c r="D35" s="4">
         <f t="shared" si="0"/>
         <v>0.77</v>
       </c>
-      <c r="E33" s="6">
+      <c r="E35" s="4">
         <f t="shared" si="3"/>
         <v>0.77</v>
       </c>
-      <c r="F33" s="6">
+      <c r="F35" s="4">
         <f t="shared" si="1"/>
         <v>0.77</v>
       </c>
-      <c r="G33" s="8" t="s">
+      <c r="G35" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="H33" s="8" t="s">
+      <c r="H35" s="6" t="s">
         <v>128</v>
       </c>
-      <c r="I33" s="10" t="s">
-        <v>210</v>
-      </c>
-      <c r="J33" s="10" t="s">
-        <v>241</v>
-      </c>
-      <c r="K33" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="L33" s="8" t="s">
+      <c r="I35" s="8" t="s">
+        <v>206</v>
+      </c>
+      <c r="J35" s="8" t="s">
+        <v>236</v>
+      </c>
+      <c r="K35" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="L35" s="6" t="s">
         <v>129</v>
       </c>
-      <c r="M33" s="8"/>
-      <c r="N33" s="7"/>
-      <c r="O33" s="8"/>
-      <c r="P33" s="5">
+      <c r="M35" s="6">
+        <v>0</v>
+      </c>
+      <c r="N35" s="5">
+        <f t="shared" si="5"/>
+        <v>46093</v>
+      </c>
+      <c r="O35" s="3">
+        <v>1</v>
+      </c>
+      <c r="P35" s="3">
         <f t="shared" si="2"/>
-        <v>-1</v>
-      </c>
-      <c r="Q33" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="Q35" s="6" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="34" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A34" s="4" t="s">
+    <row r="36" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A36" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B34" s="5">
+      <c r="B36" s="3">
         <v>2</v>
       </c>
-      <c r="C34" s="6">
+      <c r="C36" s="4">
         <v>0.1</v>
       </c>
-      <c r="D34" s="6">
+      <c r="D36" s="4">
         <f t="shared" si="0"/>
         <v>0.2</v>
       </c>
-      <c r="E34" s="6">
+      <c r="E36" s="4">
         <f t="shared" si="3"/>
         <v>0.1</v>
       </c>
-      <c r="F34" s="6">
+      <c r="F36" s="4">
         <f t="shared" si="1"/>
         <v>0.2</v>
       </c>
-      <c r="G34" s="8" t="s">
+      <c r="G36" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="H34" s="8" t="s">
-        <v>258</v>
-      </c>
-      <c r="I34" s="10" t="s">
-        <v>259</v>
-      </c>
-      <c r="J34" s="10" t="s">
-        <v>260</v>
-      </c>
-      <c r="K34" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="L34" s="8" t="s">
-        <v>261</v>
-      </c>
-      <c r="M34" s="8"/>
-      <c r="N34" s="7"/>
-      <c r="O34" s="8"/>
-      <c r="P34" s="5">
+      <c r="H36" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="I36" s="8" t="s">
+        <v>254</v>
+      </c>
+      <c r="J36" s="8" t="s">
+        <v>255</v>
+      </c>
+      <c r="K36" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="L36" s="6" t="s">
+        <v>256</v>
+      </c>
+      <c r="M36" s="6">
+        <v>0</v>
+      </c>
+      <c r="N36" s="5">
+        <f t="shared" si="5"/>
+        <v>46093</v>
+      </c>
+      <c r="O36" s="3">
+        <v>2</v>
+      </c>
+      <c r="P36" s="3">
         <f t="shared" si="2"/>
-        <v>-2</v>
-      </c>
-      <c r="Q34" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="Q36" s="6" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="35" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A35" s="4" t="s">
-        <v>160</v>
-      </c>
-      <c r="B35" s="5">
-        <v>1</v>
-      </c>
-      <c r="C35" s="6">
+    <row r="37" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A37" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="B37" s="3">
+        <v>1</v>
+      </c>
+      <c r="C37" s="4">
         <v>0.46</v>
       </c>
-      <c r="D35" s="6">
+      <c r="D37" s="4">
         <f t="shared" si="0"/>
         <v>0.46</v>
       </c>
-      <c r="E35" s="6">
+      <c r="E37" s="4">
         <f t="shared" si="3"/>
         <v>0.46</v>
       </c>
-      <c r="F35" s="6">
+      <c r="F37" s="4">
         <f t="shared" si="1"/>
         <v>0.46</v>
       </c>
-      <c r="G35" s="8" t="s">
-        <v>162</v>
-      </c>
-      <c r="H35" s="8" t="s">
-        <v>161</v>
-      </c>
-      <c r="I35" s="10" t="s">
-        <v>211</v>
-      </c>
-      <c r="J35" s="10" t="s">
-        <v>242</v>
-      </c>
-      <c r="K35" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="L35" s="8" t="s">
-        <v>163</v>
-      </c>
-      <c r="M35" s="8"/>
-      <c r="N35" s="7"/>
-      <c r="O35" s="8"/>
-      <c r="P35" s="5">
+      <c r="G37" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="H37" s="6" t="s">
+        <v>158</v>
+      </c>
+      <c r="I37" s="8" t="s">
+        <v>207</v>
+      </c>
+      <c r="J37" s="8" t="s">
+        <v>237</v>
+      </c>
+      <c r="K37" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="L37" s="6" t="s">
+        <v>160</v>
+      </c>
+      <c r="M37" s="6">
+        <v>1</v>
+      </c>
+      <c r="N37" s="5">
+        <f t="shared" si="5"/>
+        <v>46093</v>
+      </c>
+      <c r="O37" s="3">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="P37" s="3">
         <f t="shared" si="2"/>
-        <v>-1</v>
-      </c>
-      <c r="Q35" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="Q37" s="6" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="36" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A36" s="4" t="s">
-        <v>168</v>
-      </c>
-      <c r="B36" s="5">
+    <row r="38" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A38" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="B38" s="3">
         <v>3</v>
       </c>
-      <c r="C36" s="6">
+      <c r="C38" s="4">
         <v>3.55</v>
       </c>
-      <c r="D36" s="6">
+      <c r="D38" s="4">
         <f t="shared" si="0"/>
         <v>10.649999999999999</v>
       </c>
-      <c r="E36" s="6">
+      <c r="E38" s="4">
         <f t="shared" si="3"/>
         <v>3.55</v>
       </c>
-      <c r="F36" s="6">
+      <c r="F38" s="4">
         <f t="shared" si="1"/>
         <v>10.649999999999999</v>
       </c>
-      <c r="G36" s="8" t="s">
-        <v>169</v>
-      </c>
-      <c r="H36" s="8" t="s">
-        <v>170</v>
-      </c>
-      <c r="I36" s="10" t="s">
-        <v>212</v>
-      </c>
-      <c r="J36" s="10" t="s">
-        <v>243</v>
-      </c>
-      <c r="K36" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="L36" s="8" t="s">
-        <v>171</v>
-      </c>
-      <c r="M36" s="8"/>
-      <c r="N36" s="7"/>
-      <c r="O36" s="8"/>
-      <c r="P36" s="5">
+      <c r="G38" s="6" t="s">
+        <v>166</v>
+      </c>
+      <c r="H38" s="6" t="s">
+        <v>167</v>
+      </c>
+      <c r="I38" s="8" t="s">
+        <v>208</v>
+      </c>
+      <c r="J38" s="8" t="s">
+        <v>238</v>
+      </c>
+      <c r="K38" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="L38" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="M38" s="6"/>
+      <c r="N38" s="5">
+        <f t="shared" si="5"/>
+        <v>46093</v>
+      </c>
+      <c r="O38" s="3">
+        <v>3</v>
+      </c>
+      <c r="P38" s="3">
         <f t="shared" si="2"/>
-        <v>-3</v>
-      </c>
-      <c r="Q36" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="Q38" s="6" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="37" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A37" s="4" t="s">
+    <row r="39" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A39" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="B37" s="5">
-        <v>1</v>
-      </c>
-      <c r="C37" s="6">
+      <c r="B39" s="3">
+        <v>1</v>
+      </c>
+      <c r="C39" s="4">
         <v>3.77</v>
       </c>
-      <c r="D37" s="6">
+      <c r="D39" s="4">
         <f t="shared" si="0"/>
         <v>3.77</v>
       </c>
-      <c r="E37" s="6">
+      <c r="E39" s="4">
         <f t="shared" si="3"/>
         <v>3.77</v>
       </c>
-      <c r="F37" s="6">
+      <c r="F39" s="4">
         <f t="shared" si="1"/>
         <v>3.77</v>
       </c>
-      <c r="G37" s="8" t="s">
+      <c r="G39" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="H37" s="8" t="s">
+      <c r="H39" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="I37" s="10" t="s">
-        <v>213</v>
-      </c>
-      <c r="J37" s="10" t="s">
-        <v>244</v>
-      </c>
-      <c r="K37" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="L37" s="8" t="s">
+      <c r="I39" s="8" t="s">
+        <v>209</v>
+      </c>
+      <c r="J39" s="8" t="s">
+        <v>239</v>
+      </c>
+      <c r="K39" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="L39" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="M37" s="8"/>
-      <c r="N37" s="7"/>
-      <c r="O37" s="8"/>
-      <c r="P37" s="5">
+      <c r="M39" s="6">
+        <v>2</v>
+      </c>
+      <c r="N39" s="5">
+        <f t="shared" si="5"/>
+        <v>46093</v>
+      </c>
+      <c r="O39" s="3">
+        <f t="shared" si="4"/>
+        <v>2</v>
+      </c>
+      <c r="P39" s="3">
         <f t="shared" si="2"/>
-        <v>-1</v>
-      </c>
-      <c r="Q37" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="Q39" s="6" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="38" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A38" s="4" t="s">
+    <row r="40" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A40" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="B38" s="5">
-        <v>1</v>
-      </c>
-      <c r="C38" s="6">
+      <c r="B40" s="3">
+        <v>1</v>
+      </c>
+      <c r="C40" s="4">
         <v>0.71</v>
       </c>
-      <c r="D38" s="6">
+      <c r="D40" s="4">
         <f t="shared" si="0"/>
         <v>0.71</v>
       </c>
-      <c r="E38" s="6">
+      <c r="E40" s="4">
         <f t="shared" si="3"/>
         <v>0.71</v>
       </c>
-      <c r="F38" s="6">
+      <c r="F40" s="4">
         <f t="shared" si="1"/>
         <v>0.71</v>
       </c>
-      <c r="G38" s="8" t="s">
+      <c r="G40" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="H38" s="8" t="s">
+      <c r="H40" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="I38" s="10" t="s">
-        <v>214</v>
-      </c>
-      <c r="J38" s="10" t="s">
-        <v>245</v>
-      </c>
-      <c r="K38" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="L38" s="8" t="s">
+      <c r="I40" s="8" t="s">
+        <v>210</v>
+      </c>
+      <c r="J40" s="8" t="s">
+        <v>240</v>
+      </c>
+      <c r="K40" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="L40" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="M38" s="8"/>
-      <c r="N38" s="7"/>
-      <c r="O38" s="8"/>
-      <c r="P38" s="5">
+      <c r="M40" s="6">
+        <v>2</v>
+      </c>
+      <c r="N40" s="5">
+        <f t="shared" si="5"/>
+        <v>46093</v>
+      </c>
+      <c r="O40" s="3">
+        <f t="shared" si="4"/>
+        <v>2</v>
+      </c>
+      <c r="P40" s="3">
         <f t="shared" si="2"/>
-        <v>-1</v>
-      </c>
-      <c r="Q38" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="Q40" s="6" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="39" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="4" t="s">
+    <row r="41" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A41" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="B39" s="5">
+      <c r="B41" s="3">
         <v>2</v>
       </c>
-      <c r="C39" s="6">
+      <c r="C41" s="4">
         <v>0.71</v>
       </c>
-      <c r="D39" s="6">
-        <f t="shared" ref="D39:D40" si="8">B39*C39</f>
+      <c r="D41" s="4">
+        <f t="shared" ref="D41:D42" si="12">B41*C41</f>
         <v>1.42</v>
       </c>
-      <c r="E39" s="6">
-        <f t="shared" ref="E39:E40" si="9">C39</f>
+      <c r="E41" s="4">
+        <f t="shared" ref="E41:E42" si="13">C41</f>
         <v>0.71</v>
       </c>
-      <c r="F39" s="6">
-        <f t="shared" ref="F39:F40" si="10">B39*E39</f>
+      <c r="F41" s="4">
+        <f t="shared" ref="F41:F42" si="14">B41*E41</f>
         <v>1.42</v>
       </c>
-      <c r="G39" s="8" t="s">
+      <c r="G41" s="6" t="s">
         <v>132</v>
       </c>
-      <c r="H39" s="8" t="s">
+      <c r="H41" s="6" t="s">
         <v>133</v>
       </c>
-      <c r="I39" s="10" t="s">
-        <v>215</v>
-      </c>
-      <c r="J39" s="10" t="s">
-        <v>246</v>
-      </c>
-      <c r="K39" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="L39" s="8" t="s">
+      <c r="I41" s="8" t="s">
+        <v>211</v>
+      </c>
+      <c r="J41" s="8" t="s">
+        <v>241</v>
+      </c>
+      <c r="K41" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="L41" s="6" t="s">
         <v>134</v>
       </c>
-      <c r="M39" s="8"/>
-      <c r="N39" s="8"/>
-      <c r="O39" s="8"/>
-      <c r="P39" s="5">
+      <c r="M41" s="6">
+        <v>2</v>
+      </c>
+      <c r="N41" s="5">
+        <f t="shared" si="5"/>
+        <v>46093</v>
+      </c>
+      <c r="O41" s="3">
+        <f t="shared" si="4"/>
+        <v>2</v>
+      </c>
+      <c r="P41" s="3">
         <f t="shared" si="2"/>
-        <v>-2</v>
-      </c>
-      <c r="Q39" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="Q41" s="6" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="40" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="4" t="s">
+    <row r="42" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A42" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="B40" s="5">
+      <c r="B42" s="3">
         <v>3</v>
       </c>
-      <c r="C40" s="6">
+      <c r="C42" s="4">
         <v>0.32</v>
       </c>
-      <c r="D40" s="6">
-        <f t="shared" si="8"/>
+      <c r="D42" s="4">
+        <f t="shared" si="12"/>
         <v>0.96</v>
       </c>
-      <c r="E40" s="6">
-        <f t="shared" si="9"/>
+      <c r="E42" s="4">
+        <f t="shared" si="13"/>
         <v>0.32</v>
       </c>
-      <c r="F40" s="6">
-        <f t="shared" si="10"/>
+      <c r="F42" s="4">
+        <f t="shared" si="14"/>
         <v>0.96</v>
       </c>
-      <c r="G40" s="8" t="s">
+      <c r="G42" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="H40" s="8" t="s">
+      <c r="H42" s="6" t="s">
         <v>135</v>
       </c>
-      <c r="I40" s="10" t="s">
-        <v>216</v>
-      </c>
-      <c r="J40" s="10" t="s">
-        <v>247</v>
-      </c>
-      <c r="K40" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="L40" s="8" t="s">
+      <c r="I42" s="8" t="s">
+        <v>212</v>
+      </c>
+      <c r="J42" s="8" t="s">
+        <v>242</v>
+      </c>
+      <c r="K42" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="L42" s="6" t="s">
         <v>136</v>
       </c>
-      <c r="M40" s="8"/>
-      <c r="N40" s="8"/>
-      <c r="O40" s="8"/>
-      <c r="P40" s="5">
+      <c r="M42" s="6">
+        <v>0</v>
+      </c>
+      <c r="N42" s="5">
+        <f t="shared" si="5"/>
+        <v>46093</v>
+      </c>
+      <c r="O42" s="3">
+        <v>3</v>
+      </c>
+      <c r="P42" s="3">
         <f t="shared" si="2"/>
-        <v>-3</v>
-      </c>
-      <c r="Q40" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="Q42" s="6" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="41" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C41" s="8" t="s">
+    <row r="43" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C43" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="D41" s="9">
-        <f t="shared" ref="D40:D41" si="11">SUM(D5:D40)</f>
-        <v>78.63</v>
-      </c>
-      <c r="E41" s="8" t="s">
+      <c r="D43" s="7">
+        <f>SUM(D5:D42)</f>
+        <v>87.089999999999975</v>
+      </c>
+      <c r="E43" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="F41" s="9">
-        <f t="shared" ref="F40:F41" si="12">SUM(F5:F40)</f>
-        <v>78.63</v>
+      <c r="F43" s="7">
+        <f t="shared" ref="F43" si="15">SUM(F5:F42)</f>
+        <v>87.089999999999975</v>
       </c>
     </row>
   </sheetData>
@@ -3327,65 +3780,63 @@
     <hyperlink ref="I19" r:id="rId17" xr:uid="{B623BDED-D003-434D-8040-DD0F98055F8E}"/>
     <hyperlink ref="I20" r:id="rId18" xr:uid="{3A2131FD-4733-40D7-BB54-2A09C2CC2323}"/>
     <hyperlink ref="I21" r:id="rId19" xr:uid="{9911FEA8-F68A-4C34-A23E-DFDF3F5F52C4}"/>
-    <hyperlink ref="I22" r:id="rId20" xr:uid="{DBF00FE0-2343-40E8-8945-5E999EDD6AFE}"/>
-    <hyperlink ref="I23" r:id="rId21" xr:uid="{89CAEAEF-8126-4E70-8DA1-F8BB6653A191}"/>
-    <hyperlink ref="I24" r:id="rId22" xr:uid="{23D1E758-5C38-4BC7-BA64-58FD8C08DC2B}"/>
-    <hyperlink ref="I25" r:id="rId23" xr:uid="{12927891-2EB0-4C68-83BC-0E6C97C5E4F0}"/>
-    <hyperlink ref="I26" r:id="rId24" xr:uid="{3F274505-DBA4-43B7-9558-13DB281033DC}"/>
-    <hyperlink ref="I27" r:id="rId25" xr:uid="{5C394CA1-5313-4D38-A861-E50D40D505CC}"/>
-    <hyperlink ref="I28" r:id="rId26" xr:uid="{42A7CC4D-85DE-4AD2-9382-C0EB45C1C95C}"/>
-    <hyperlink ref="I29" r:id="rId27" xr:uid="{25181389-4B87-4586-A97C-0A8CB3A5E179}"/>
-    <hyperlink ref="I32" r:id="rId28" xr:uid="{C7DD35A4-ED9D-4C69-B301-607A86192B8E}"/>
-    <hyperlink ref="I33" r:id="rId29" xr:uid="{C4B1ED7A-D46B-4433-8E18-7C43597A43FC}"/>
-    <hyperlink ref="I35" r:id="rId30" xr:uid="{8C1FA9AB-BF98-48CE-A151-19BEE682DBEA}"/>
-    <hyperlink ref="I36" r:id="rId31" xr:uid="{4A7FAC4D-9D62-4B68-AA2D-5BCA9EC77F29}"/>
-    <hyperlink ref="I37" r:id="rId32" xr:uid="{00CD0ED5-4C61-4A08-9F6A-5CFF3B75A7A4}"/>
-    <hyperlink ref="I38" r:id="rId33" xr:uid="{40788476-2F32-458C-BD69-FC4E1967E209}"/>
-    <hyperlink ref="I39" r:id="rId34" xr:uid="{F34B2D45-372F-4200-A1E4-168FBFD1BE75}"/>
-    <hyperlink ref="I40" r:id="rId35" xr:uid="{64E4C49D-2401-4763-B23B-F38BAC3E98FD}"/>
-    <hyperlink ref="J3" r:id="rId36" xr:uid="{AE5C57B0-3975-49A0-9F10-867BFF0C511A}"/>
-    <hyperlink ref="J4" r:id="rId37" xr:uid="{C9B7A6DB-8BF0-4D84-80C1-7F7ECC52AFBD}"/>
-    <hyperlink ref="J5" r:id="rId38" xr:uid="{E469D8A1-7025-4DEE-B057-9290EC969475}"/>
-    <hyperlink ref="J6" r:id="rId39" xr:uid="{C9DDB307-618C-4E05-8640-376D139B93EF}"/>
-    <hyperlink ref="J7" r:id="rId40" xr:uid="{59E4D5DC-69FA-4F37-AAAF-4207DC87FF99}"/>
-    <hyperlink ref="J8" r:id="rId41" xr:uid="{FA2F61BB-B5EC-4CAC-8A7E-A00301B969A7}"/>
-    <hyperlink ref="J9" r:id="rId42" xr:uid="{92035C51-830F-47A3-9AF7-25115EF5A4CA}"/>
-    <hyperlink ref="J10" r:id="rId43" xr:uid="{B95AC53F-FFD8-4526-B7C3-0A5EEDE7D1B2}"/>
-    <hyperlink ref="J11" r:id="rId44" xr:uid="{94374666-9511-4B34-A2CB-6F3EF5A767EC}"/>
-    <hyperlink ref="J12" r:id="rId45" xr:uid="{9A4CEB44-D505-407C-B5A6-7B3280A0B33B}"/>
-    <hyperlink ref="J13" r:id="rId46" xr:uid="{0E50E3BC-2C9A-4872-A410-AA9D7DB9C199}"/>
-    <hyperlink ref="J14" r:id="rId47" xr:uid="{06DB70E1-456D-4EAB-938C-BAF6D676CE10}"/>
-    <hyperlink ref="J15" r:id="rId48" xr:uid="{8CF0CD79-EB8A-4E6D-B3A7-D6E2DA4069F7}"/>
-    <hyperlink ref="J16" r:id="rId49" xr:uid="{1C31C9CC-5DAB-4BAA-986D-34DA2ECDDDCF}"/>
-    <hyperlink ref="J17" r:id="rId50" xr:uid="{FC42D22D-4BE4-4AE6-9381-858BB598A0E0}"/>
-    <hyperlink ref="J18" r:id="rId51" xr:uid="{E9FAB5B9-B37A-4282-A75B-4F9B75D55796}"/>
-    <hyperlink ref="J19" r:id="rId52" xr:uid="{E877F378-04D2-443A-B3A6-72281D32377A}"/>
-    <hyperlink ref="J20" r:id="rId53" xr:uid="{ADBD8819-49C5-46D8-AD00-AB3BDEEA0D9D}"/>
-    <hyperlink ref="J21" r:id="rId54" xr:uid="{FE1613F9-5D8C-4A9E-B7AD-A94D9E839B37}"/>
-    <hyperlink ref="J22" r:id="rId55" xr:uid="{8827A2D9-D128-446F-ACFF-D4EDAB5AD250}"/>
-    <hyperlink ref="J23" r:id="rId56" xr:uid="{B5DB80EE-F028-4749-94EC-5DFE122AA3A9}"/>
-    <hyperlink ref="J24" r:id="rId57" xr:uid="{CBD26CC1-92E2-4210-AA6D-B84B9B6E9FAC}"/>
-    <hyperlink ref="J25" r:id="rId58" xr:uid="{204C57B2-24F0-4924-9838-CFDCF7064F11}"/>
-    <hyperlink ref="J26" r:id="rId59" xr:uid="{0FD0A0B4-A620-4D6A-8D8F-A7E644F1947D}"/>
-    <hyperlink ref="J27" r:id="rId60" xr:uid="{60C096EB-20ED-4C54-A5B3-F804B5DDAFB7}"/>
-    <hyperlink ref="J28" r:id="rId61" xr:uid="{1C64A966-AC83-4C05-8F0B-18A2DA80EA56}"/>
-    <hyperlink ref="J29" r:id="rId62" xr:uid="{BF1B5A6B-D2E5-4396-A058-445A47D7EDA5}"/>
-    <hyperlink ref="J33" r:id="rId63" xr:uid="{B81519DB-E70A-43DD-8BA4-18A7D7AD6B11}"/>
-    <hyperlink ref="J35" r:id="rId64" xr:uid="{56802FE4-F16D-4E08-AA6A-D24690C2321A}"/>
-    <hyperlink ref="J36" r:id="rId65" xr:uid="{A862BCF8-0D68-455C-8D8D-D5D89F406DB8}"/>
-    <hyperlink ref="J37" r:id="rId66" xr:uid="{C3D07864-52C5-4E04-8DA8-80A8AE130A87}"/>
-    <hyperlink ref="J38" r:id="rId67" xr:uid="{D35109BC-4B9B-4629-B88C-59DC2DD8566D}"/>
-    <hyperlink ref="J39" r:id="rId68" xr:uid="{2322B1B5-C5A3-4E94-8003-BD6B32BC1CF4}"/>
-    <hyperlink ref="J40" r:id="rId69" xr:uid="{DE2905BA-86A4-49B3-88C1-05462AF53A80}"/>
-    <hyperlink ref="I30" r:id="rId70" xr:uid="{DC73759F-3FDD-420E-B89A-7A9952898676}"/>
-    <hyperlink ref="J32" r:id="rId71" xr:uid="{FF4E4D84-DA5F-4193-BF3C-776B33129549}"/>
-    <hyperlink ref="J31" r:id="rId72" xr:uid="{2D4A5CFC-0649-431C-8058-4038507C75EE}"/>
-    <hyperlink ref="I31" r:id="rId73" xr:uid="{DF76FD57-D796-4392-8BE0-DFB239421522}"/>
-    <hyperlink ref="J30" r:id="rId74" xr:uid="{88BC990B-7AF1-4EC1-A6D9-04F317EBAD33}"/>
-    <hyperlink ref="I34" r:id="rId75" display="https://www.digikey.com/en/products/detail/same-sky-formerly-cui-devices-/TS02-66-55-BK-100-LCR-D/15634297?gclsrc=aw.ds&amp;gad_source=1&amp;gad_campaignid=21273973101&amp;gbraid=0AAAAADrbLliDycjgJofPVWAUnaFDHZ4Dd&amp;gclid=Cj0KCQiA8KTNBhD_ARIsAOvp6DJm3WPshQnES_nFbYzMUKpoAK0on-aVhdqwQv7LWtPFiyFmBonGw60aAhTiEALw_wcB " xr:uid="{E1A08DAF-AECF-4592-BA50-775441E5921C}"/>
-    <hyperlink ref="J34" r:id="rId76" xr:uid="{B73BC35A-3897-4F61-B017-5964ACFB946C}"/>
+    <hyperlink ref="I24" r:id="rId20" xr:uid="{DBF00FE0-2343-40E8-8945-5E999EDD6AFE}"/>
+    <hyperlink ref="I25" r:id="rId21" xr:uid="{89CAEAEF-8126-4E70-8DA1-F8BB6653A191}"/>
+    <hyperlink ref="I26" r:id="rId22" xr:uid="{23D1E758-5C38-4BC7-BA64-58FD8C08DC2B}"/>
+    <hyperlink ref="I27" r:id="rId23" xr:uid="{12927891-2EB0-4C68-83BC-0E6C97C5E4F0}"/>
+    <hyperlink ref="I29" r:id="rId24" xr:uid="{5C394CA1-5313-4D38-A861-E50D40D505CC}"/>
+    <hyperlink ref="I30" r:id="rId25" xr:uid="{42A7CC4D-85DE-4AD2-9382-C0EB45C1C95C}"/>
+    <hyperlink ref="I31" r:id="rId26" xr:uid="{25181389-4B87-4586-A97C-0A8CB3A5E179}"/>
+    <hyperlink ref="I34" r:id="rId27" xr:uid="{C7DD35A4-ED9D-4C69-B301-607A86192B8E}"/>
+    <hyperlink ref="I35" r:id="rId28" xr:uid="{C4B1ED7A-D46B-4433-8E18-7C43597A43FC}"/>
+    <hyperlink ref="I37" r:id="rId29" xr:uid="{8C1FA9AB-BF98-48CE-A151-19BEE682DBEA}"/>
+    <hyperlink ref="I38" r:id="rId30" xr:uid="{4A7FAC4D-9D62-4B68-AA2D-5BCA9EC77F29}"/>
+    <hyperlink ref="I39" r:id="rId31" xr:uid="{00CD0ED5-4C61-4A08-9F6A-5CFF3B75A7A4}"/>
+    <hyperlink ref="I40" r:id="rId32" xr:uid="{40788476-2F32-458C-BD69-FC4E1967E209}"/>
+    <hyperlink ref="I41" r:id="rId33" xr:uid="{F34B2D45-372F-4200-A1E4-168FBFD1BE75}"/>
+    <hyperlink ref="I42" r:id="rId34" xr:uid="{64E4C49D-2401-4763-B23B-F38BAC3E98FD}"/>
+    <hyperlink ref="J3" r:id="rId35" xr:uid="{AE5C57B0-3975-49A0-9F10-867BFF0C511A}"/>
+    <hyperlink ref="J4" r:id="rId36" xr:uid="{C9B7A6DB-8BF0-4D84-80C1-7F7ECC52AFBD}"/>
+    <hyperlink ref="J5" r:id="rId37" xr:uid="{E469D8A1-7025-4DEE-B057-9290EC969475}"/>
+    <hyperlink ref="J6" r:id="rId38" xr:uid="{C9DDB307-618C-4E05-8640-376D139B93EF}"/>
+    <hyperlink ref="J7" r:id="rId39" xr:uid="{59E4D5DC-69FA-4F37-AAAF-4207DC87FF99}"/>
+    <hyperlink ref="J8" r:id="rId40" xr:uid="{FA2F61BB-B5EC-4CAC-8A7E-A00301B969A7}"/>
+    <hyperlink ref="J9" r:id="rId41" xr:uid="{92035C51-830F-47A3-9AF7-25115EF5A4CA}"/>
+    <hyperlink ref="J10" r:id="rId42" xr:uid="{B95AC53F-FFD8-4526-B7C3-0A5EEDE7D1B2}"/>
+    <hyperlink ref="J11" r:id="rId43" xr:uid="{94374666-9511-4B34-A2CB-6F3EF5A767EC}"/>
+    <hyperlink ref="J12" r:id="rId44" xr:uid="{9A4CEB44-D505-407C-B5A6-7B3280A0B33B}"/>
+    <hyperlink ref="J13" r:id="rId45" xr:uid="{0E50E3BC-2C9A-4872-A410-AA9D7DB9C199}"/>
+    <hyperlink ref="J14" r:id="rId46" xr:uid="{06DB70E1-456D-4EAB-938C-BAF6D676CE10}"/>
+    <hyperlink ref="J15" r:id="rId47" xr:uid="{8CF0CD79-EB8A-4E6D-B3A7-D6E2DA4069F7}"/>
+    <hyperlink ref="J16" r:id="rId48" xr:uid="{1C31C9CC-5DAB-4BAA-986D-34DA2ECDDDCF}"/>
+    <hyperlink ref="J17" r:id="rId49" xr:uid="{FC42D22D-4BE4-4AE6-9381-858BB598A0E0}"/>
+    <hyperlink ref="J18" r:id="rId50" xr:uid="{E9FAB5B9-B37A-4282-A75B-4F9B75D55796}"/>
+    <hyperlink ref="J19" r:id="rId51" xr:uid="{E877F378-04D2-443A-B3A6-72281D32377A}"/>
+    <hyperlink ref="J20" r:id="rId52" xr:uid="{ADBD8819-49C5-46D8-AD00-AB3BDEEA0D9D}"/>
+    <hyperlink ref="J21" r:id="rId53" xr:uid="{FE1613F9-5D8C-4A9E-B7AD-A94D9E839B37}"/>
+    <hyperlink ref="J24" r:id="rId54" xr:uid="{8827A2D9-D128-446F-ACFF-D4EDAB5AD250}"/>
+    <hyperlink ref="J25" r:id="rId55" xr:uid="{B5DB80EE-F028-4749-94EC-5DFE122AA3A9}"/>
+    <hyperlink ref="J26" r:id="rId56" xr:uid="{CBD26CC1-92E2-4210-AA6D-B84B9B6E9FAC}"/>
+    <hyperlink ref="J27" r:id="rId57" xr:uid="{204C57B2-24F0-4924-9838-CFDCF7064F11}"/>
+    <hyperlink ref="J29" r:id="rId58" xr:uid="{60C096EB-20ED-4C54-A5B3-F804B5DDAFB7}"/>
+    <hyperlink ref="J30" r:id="rId59" xr:uid="{1C64A966-AC83-4C05-8F0B-18A2DA80EA56}"/>
+    <hyperlink ref="J31" r:id="rId60" xr:uid="{BF1B5A6B-D2E5-4396-A058-445A47D7EDA5}"/>
+    <hyperlink ref="J35" r:id="rId61" xr:uid="{B81519DB-E70A-43DD-8BA4-18A7D7AD6B11}"/>
+    <hyperlink ref="J37" r:id="rId62" xr:uid="{56802FE4-F16D-4E08-AA6A-D24690C2321A}"/>
+    <hyperlink ref="J38" r:id="rId63" xr:uid="{A862BCF8-0D68-455C-8D8D-D5D89F406DB8}"/>
+    <hyperlink ref="J39" r:id="rId64" xr:uid="{C3D07864-52C5-4E04-8DA8-80A8AE130A87}"/>
+    <hyperlink ref="J40" r:id="rId65" xr:uid="{D35109BC-4B9B-4629-B88C-59DC2DD8566D}"/>
+    <hyperlink ref="J41" r:id="rId66" xr:uid="{2322B1B5-C5A3-4E94-8003-BD6B32BC1CF4}"/>
+    <hyperlink ref="J42" r:id="rId67" xr:uid="{DE2905BA-86A4-49B3-88C1-05462AF53A80}"/>
+    <hyperlink ref="I32" r:id="rId68" xr:uid="{DC73759F-3FDD-420E-B89A-7A9952898676}"/>
+    <hyperlink ref="J34" r:id="rId69" xr:uid="{FF4E4D84-DA5F-4193-BF3C-776B33129549}"/>
+    <hyperlink ref="J33" r:id="rId70" xr:uid="{2D4A5CFC-0649-431C-8058-4038507C75EE}"/>
+    <hyperlink ref="I33" r:id="rId71" xr:uid="{DF76FD57-D796-4392-8BE0-DFB239421522}"/>
+    <hyperlink ref="J32" r:id="rId72" xr:uid="{88BC990B-7AF1-4EC1-A6D9-04F317EBAD33}"/>
+    <hyperlink ref="I36" r:id="rId73" display="https://www.digikey.com/en/products/detail/same-sky-formerly-cui-devices-/TS02-66-55-BK-100-LCR-D/15634297?gclsrc=aw.ds&amp;gad_source=1&amp;gad_campaignid=21273973101&amp;gbraid=0AAAAADrbLliDycjgJofPVWAUnaFDHZ4Dd&amp;gclid=Cj0KCQiA8KTNBhD_ARIsAOvp6DJm3WPshQnES_nFbYzMUKpoAK0on-aVhdqwQv7LWtPFiyFmBonGw60aAhTiEALw_wcB " xr:uid="{E1A08DAF-AECF-4592-BA50-775441E5921C}"/>
+    <hyperlink ref="J36" r:id="rId74" xr:uid="{B73BC35A-3897-4F61-B017-5964ACFB946C}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="landscape" r:id="rId77"/>
+  <pageSetup orientation="landscape" r:id="rId75"/>
 </worksheet>
 </file>
</xml_diff>